<commit_message>
POCOR-3533 - Improve on logic to check for principal and homeroom teacher edit comments for report cards
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16060" tabRatio="500" activeTab="2"/>
+    <workbookView xWindow="8600" yWindow="1380" windowWidth="25600" windowHeight="16060" tabRatio="500" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="24" r:id="rId1"/>
@@ -158,9 +158,6 @@
     <t>${"match": {"displayValue": "InstitutionStudentsReportCardsComments.comments","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "InstitutionStudentsReportCardsComments.education_subject_id"}}}</t>
   </si>
   <si>
-    <t>${"match": {"displayValue": "AssessmentItemResults.marks_formatted","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "AssessmentItemResults.education_subject_id"},"columns": {"matchFrom": "AssessmentPeriods.id","matchTo": "AssessmentItemResults.assessment_period_id"}}}</t>
-  </si>
-  <si>
     <t>${"repeatRows":{"displayValue":"AssessmentItems.education_subject.name"}}</t>
   </si>
   <si>
@@ -219,6 +216,9 @@
   </si>
   <si>
     <t>${"match": {"displayValue": "InstitutionStudentsReportCardsComments.comment_code_name","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "InstitutionStudentsReportCardsComments.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "AssessmentItemResults.marks_formatted","type":"number","format":"2","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "AssessmentItemResults.education_subject_id"},"columns": {"matchFrom": "AssessmentPeriods.id","matchTo": "AssessmentItemResults.assessment_period_id"}}}</t>
   </si>
 </sst>
 </file>
@@ -614,6 +614,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -639,9 +642,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1192,7 +1192,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="26"/>
+      <c r="A1" s="27"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
       <c r="D1" s="1"/>
@@ -1201,10 +1201,10 @@
       <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:7" ht="26" customHeight="1">
-      <c r="A2" s="26"/>
+      <c r="A2" s="27"/>
       <c r="B2" s="1"/>
       <c r="C2" s="34" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D2" s="34"/>
       <c r="E2" s="34"/>
@@ -1212,7 +1212,7 @@
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" ht="23" customHeight="1">
-      <c r="A3" s="26"/>
+      <c r="A3" s="27"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1233,15 +1233,15 @@
       <c r="A5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="33"/>
+      <c r="C5" s="24"/>
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="9"/>
@@ -1250,15 +1250,15 @@
       <c r="A6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="33" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" s="33"/>
+      <c r="B6" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="24"/>
       <c r="D6" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="9"/>
@@ -1267,15 +1267,15 @@
       <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="32"/>
+      <c r="C7" s="33"/>
       <c r="D7" s="6" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F7" s="8"/>
       <c r="G7" s="9"/>
@@ -1284,15 +1284,15 @@
       <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="32"/>
+      <c r="C8" s="33"/>
       <c r="D8" s="6" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F8" s="8"/>
       <c r="G8" s="9"/>
@@ -1301,10 +1301,10 @@
       <c r="A9" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="33"/>
+      <c r="C9" s="24"/>
       <c r="D9" s="6" t="s">
         <v>1</v>
       </c>
@@ -1324,21 +1324,21 @@
       <c r="G10" s="10"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="30"/>
-      <c r="C11" s="30"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
       <c r="F11" s="11"/>
       <c r="G11" s="11"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="24"/>
+      <c r="B12" s="25"/>
       <c r="C12" s="12" t="s">
         <v>23</v>
       </c>
@@ -1348,10 +1348,10 @@
       <c r="G12" s="13"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="24"/>
+      <c r="B13" s="25"/>
       <c r="C13" s="12" t="s">
         <v>25</v>
       </c>
@@ -1361,10 +1361,10 @@
       <c r="G13" s="13"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="24"/>
+      <c r="B14" s="25"/>
       <c r="C14" s="12" t="s">
         <v>27</v>
       </c>
@@ -1383,15 +1383,15 @@
       <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="29"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="30"/>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="15" t="s">
@@ -1401,10 +1401,10 @@
         <v>35</v>
       </c>
       <c r="C17" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D17" s="15" t="s">
         <v>63</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>64</v>
       </c>
       <c r="E17" s="15" t="s">
         <v>36</v>
@@ -1433,10 +1433,10 @@
         <v>43</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16" customHeight="1">
@@ -1449,61 +1449,61 @@
       <c r="G19" s="10"/>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="29"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="30"/>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="24" t="s">
+      <c r="A21" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="25" t="s">
+      <c r="B21" s="25"/>
+      <c r="C21" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="24" t="s">
+      <c r="A22" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="24"/>
-      <c r="C22" s="25" t="s">
+      <c r="B22" s="25"/>
+      <c r="C22" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C22:G22"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="C2:F2"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="A20:G20"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
@@ -1531,13 +1531,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="16" t="s">
@@ -1558,13 +1558,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
       <c r="E3" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1596,7 +1596,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -1604,7 +1604,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="36" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" s="36"/>
       <c r="C2" s="36"/>
@@ -1612,27 +1612,27 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D4" s="23" t="s">
         <v>44</v>

</xml_diff>

<commit_message>
POCOR-3533 - Add total marks for report card template, fix bug on download behaviour where filetype is not correct, fix sorting for report card comments and statuses, fix subject comment tabs not showing properly, and fix finder names to camel case
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -4,13 +4,18 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="8600" yWindow="1380" windowWidth="25600" windowHeight="16060" tabRatio="500" activeTab="2"/>
+    <workbookView xWindow="13660" yWindow="900" windowWidth="22820" windowHeight="16060" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="24" r:id="rId1"/>
     <sheet name="Competencies" sheetId="16" r:id="rId2"/>
     <sheet name="Assessments" sheetId="18" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">Assessments!$A$1:$E$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Competencies!$A$1:$E$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">General!$A$1:$G$23</definedName>
+  </definedNames>
   <calcPr calcId="140000" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
@@ -21,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
   <si>
     <t>${InstitutionClasses.name}</t>
   </si>
@@ -56,9 +61,6 @@
     <t>OpenEMIS ID:</t>
   </si>
   <si>
-    <t>Prinicipal:</t>
-  </si>
-  <si>
     <t>Student:</t>
   </si>
   <si>
@@ -200,9 +202,6 @@
     <t>${"match": {"displayValue": "StudentBehaviours.time_of_behaviour","type": "time","format":"H:i:s","rows": {"matchFrom": "StudentBehaviours.id","matchTo": "StudentBehaviours.id"}}}</t>
   </si>
   <si>
-    <t>${"match": {"displayValue": "StudentBehaviours.date_of_behaviour","type": "date","format":"d-m-Y","rows": {"matchFrom": "StudentBehaviours.id","matchTo": "StudentBehaviours.id"}}}</t>
-  </si>
-  <si>
     <t>${ReportCards.academic_period.name} - ${ReportCards.name}</t>
   </si>
   <si>
@@ -219,6 +218,18 @@
   </si>
   <si>
     <t>${"match": {"displayValue": "AssessmentItemResults.marks_formatted","type":"number","format":"2","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "AssessmentItemResults.education_subject_id"},"columns": {"matchFrom": "AssessmentPeriods.id","matchTo": "AssessmentItemResults.assessment_period_id"}}}</t>
+  </si>
+  <si>
+    <t>Total Marks</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionSubjectStudents.total_mark","type":"number","format":"2","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "InstitutionSubjectStudents.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>Principal:</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "StudentBehaviours.date_of_behaviour","type": "date","format":"d/m/Y","rows": {"matchFrom": "StudentBehaviours.id","matchTo": "StudentBehaviours.id"}}}</t>
   </si>
 </sst>
 </file>
@@ -322,7 +333,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -372,15 +383,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -392,7 +394,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="153">
+  <cellStyleXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -546,8 +548,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -562,16 +568,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -596,52 +592,68 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -654,7 +666,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="153">
+  <cellStyles count="157">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -731,6 +743,8 @@
     <cellStyle name="Followed Hyperlink" xfId="148" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="150" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="152" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="154" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="156" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -807,6 +821,8 @@
     <cellStyle name="Hyperlink" xfId="147" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="149" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="151" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="153" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="155" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1187,12 +1203,14 @@
     <col min="3" max="3" width="15.83203125" style="4" customWidth="1"/>
     <col min="4" max="4" width="16" style="4" customWidth="1"/>
     <col min="5" max="5" width="28" style="4" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="10.83203125" style="4"/>
+    <col min="6" max="6" width="11.1640625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="10.5" style="4" customWidth="1"/>
+    <col min="9" max="16384" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="27"/>
+      <c r="A1" s="31"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
       <c r="D1" s="1"/>
@@ -1201,18 +1219,18 @@
       <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:7" ht="26" customHeight="1">
-      <c r="A2" s="27"/>
+      <c r="A2" s="31"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="34" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
+      <c r="C2" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" ht="23" customHeight="1">
-      <c r="A3" s="27"/>
+      <c r="A3" s="31"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1221,170 +1239,170 @@
       <c r="G3" s="3"/>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="3"/>
+      <c r="A4" s="19"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="24" t="s">
+      <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="24"/>
-      <c r="D5" s="6" t="s">
+      <c r="B5" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="C5" s="35"/>
+      <c r="D5" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="22"/>
+      <c r="G5" s="23"/>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="35"/>
+      <c r="D6" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="9"/>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="22"/>
+      <c r="G6" s="23"/>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="34"/>
+      <c r="D7" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="9"/>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="7" t="s">
+      <c r="F7" s="22"/>
+      <c r="G7" s="23"/>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="34"/>
+      <c r="D8" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="9"/>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="32" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="9"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="23"/>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="24"/>
-      <c r="D9" s="6" t="s">
+      <c r="C9" s="35"/>
+      <c r="D9" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="9"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="23"/>
     </row>
     <row r="10" spans="1:7" ht="17" customHeight="1">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="6"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="31"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="25" t="s">
+      <c r="B12" s="26"/>
+      <c r="C12" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="12" t="s">
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="25" t="s">
+      <c r="B13" s="26"/>
+      <c r="C13" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="25"/>
-      <c r="C13" s="12" t="s">
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="25" t="s">
+      <c r="B14" s="26"/>
+      <c r="C14" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7" ht="17" customHeight="1">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B16" s="29"/>
       <c r="C16" s="29"/>
@@ -1394,63 +1412,63 @@
       <c r="G16" s="30"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="C17" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="E17" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" s="15" t="s">
+      <c r="F17" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="G17" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="G17" s="15" t="s">
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="17" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="12" t="s">
+      <c r="B18" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="C18" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="D18" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="E18" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>58</v>
+      <c r="F18" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="G18" s="17" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16" customHeight="1">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="28" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B20" s="29"/>
       <c r="C20" s="29"/>
@@ -1460,30 +1478,30 @@
       <c r="G20" s="30"/>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="26"/>
+      <c r="C21" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="26" t="s">
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="25" t="s">
+      <c r="B22" s="26"/>
+      <c r="C22" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="25"/>
-      <c r="C22" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -1511,7 +1529,7 @@
   <drawing r:id="rId1"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="1" OnePage="0" WScale="0"/>
+      <mx:PLV Mode="1" OnePage="0" WScale="100"/>
     </ext>
   </extLst>
 </worksheet>
@@ -1519,53 +1537,60 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="17.5" style="4" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" style="4" customWidth="1"/>
     <col min="3" max="3" width="29" style="4" customWidth="1"/>
-    <col min="4" max="4" width="36.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="34.33203125" style="4" customWidth="1"/>
     <col min="5" max="5" width="16" style="4" customWidth="1"/>
     <col min="6" max="16384" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="16" t="s">
+      <c r="B2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="C2" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="D2" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="E2" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>20</v>
-      </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12" t="s">
-        <v>52</v>
-      </c>
+      <c r="A3" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1576,7 +1601,7 @@
   <pageSetup orientation="landscape" horizontalDpi="4294967294" verticalDpi="4294967294"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="1" OnePage="0" WScale="0"/>
+      <mx:PLV Mode="1" OnePage="0" WScale="100"/>
     </ext>
   </extLst>
 </worksheet>
@@ -1584,71 +1609,80 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <cols>
-    <col min="1" max="1" width="19.5" style="4" customWidth="1"/>
-    <col min="2" max="2" width="12.1640625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="27.33203125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="26.1640625" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="4"/>
+    <col min="1" max="1" width="16.83203125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="11.1640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="23" style="4" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" style="4" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="36" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="19" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="B3" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="C3" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" s="15" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="21" t="s">
+      <c r="E3" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="22" t="s">
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>44</v>
+      <c r="D4" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967294" verticalDpi="4294967294"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="1" OnePage="0" WScale="0"/>
+      <mx:PLV Mode="1" OnePage="0" WScale="100"/>
     </ext>
   </extLst>
 </worksheet>

</xml_diff>

<commit_message>
POCOR-4156 - Adding the BMI to the report card. - BMI only get latest record within the report card start and end date. - BMI only support institution student. - Moved the logic to count the BMI to the beforeMarshall. - Adding association to the securityUsersTable.
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="27430"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
     <workbookView xWindow="13660" yWindow="900" windowWidth="22820" windowHeight="16060" tabRatio="500"/>
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="2">Assessments!$A$1:$E$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">Competencies!$A$1:$E$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">General!$A$1:$G$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">General!$A$1:$G$25</definedName>
   </definedNames>
   <calcPr calcId="140000" concurrentCalc="0"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t>${InstitutionClasses.name}</t>
   </si>
@@ -230,6 +230,30 @@
   </si>
   <si>
     <t>${"match": {"displayValue": "StudentBehaviours.date_of_behaviour","type": "date","format":"d/m/Y","rows": {"matchFrom": "StudentBehaviours.id","matchTo": "StudentBehaviours.id"}}}</t>
+  </si>
+  <si>
+    <t>Identity Number:</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.student.identity_number}</t>
+  </si>
+  <si>
+    <t>Height:</t>
+  </si>
+  <si>
+    <t>Weight:</t>
+  </si>
+  <si>
+    <t>BMI:</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.body_mass.body_mass_index}</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.body_mass.height} m</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.body_mass.weight} kg</t>
   </si>
 </sst>
 </file>
@@ -394,7 +418,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="157">
+  <cellStyleXfs count="181">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -552,8 +576,32 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -626,39 +674,42 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -666,7 +717,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="157">
+  <cellStyles count="181">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -745,6 +796,18 @@
     <cellStyle name="Followed Hyperlink" xfId="152" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="154" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="156" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="158" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="160" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="162" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="164" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="166" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="168" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="170" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="172" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="174" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="176" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="178" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="180" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -823,6 +886,18 @@
     <cellStyle name="Hyperlink" xfId="151" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="153" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="155" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="157" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="159" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="161" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="163" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="165" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="167" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="169" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="171" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="173" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="175" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="177" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="179" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1195,7 +1270,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="16.83203125" style="4" customWidth="1"/>
@@ -1210,7 +1285,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="31"/>
+      <c r="A1" s="27"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
       <c r="D1" s="1"/>
@@ -1219,7 +1294,7 @@
       <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:7" ht="26" customHeight="1">
-      <c r="A2" s="31"/>
+      <c r="A2" s="27"/>
       <c r="B2" s="1"/>
       <c r="C2" s="36" t="s">
         <v>58</v>
@@ -1230,7 +1305,7 @@
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" ht="23" customHeight="1">
-      <c r="A3" s="31"/>
+      <c r="A3" s="27"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1290,10 +1365,10 @@
       </c>
       <c r="C7" s="34"/>
       <c r="D7" s="20" t="s">
-        <v>7</v>
+        <v>68</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="F7" s="22"/>
       <c r="G7" s="23"/>
@@ -1307,221 +1382,256 @@
       </c>
       <c r="C8" s="34"/>
       <c r="D8" s="20" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F8" s="22"/>
       <c r="G8" s="23"/>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="35" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" s="35"/>
+        <v>1</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="26"/>
       <c r="D9" s="20" t="s">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="F9" s="22"/>
       <c r="G9" s="23"/>
     </row>
-    <row r="10" spans="1:7" ht="17" customHeight="1">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="6"/>
+    <row r="10" spans="1:7">
+      <c r="A10" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="35"/>
+      <c r="D10" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="22"/>
+      <c r="G10" s="23"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="35" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" s="35"/>
+      <c r="D11" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="F11" s="22"/>
+      <c r="G11" s="23"/>
+    </row>
+    <row r="12" spans="1:7" ht="17" customHeight="1">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="6"/>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="26" t="s">
+      <c r="B13" s="32"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="8" t="s">
+      <c r="B14" s="28"/>
+      <c r="C14" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="8" t="s">
-        <v>26</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
       <c r="G14" s="9"/>
     </row>
-    <row r="15" spans="1:7" ht="17" customHeight="1">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
+    <row r="15" spans="1:7">
+      <c r="A15" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="28"/>
+      <c r="C15" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="28"/>
+      <c r="C16" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+    </row>
+    <row r="17" spans="1:7" ht="17" customHeight="1">
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="30"/>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="11" t="s">
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="31"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B19" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C19" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D19" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E19" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F19" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G19" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="17" t="s">
+    <row r="20" spans="1:7">
+      <c r="A20" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B20" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C20" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D20" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E20" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="F20" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="G18" s="17" t="s">
+      <c r="G20" s="17" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="16" customHeight="1">
-      <c r="A19" s="6"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="28" t="s">
+    <row r="21" spans="1:7" ht="16" customHeight="1">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="30"/>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="26" t="s">
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="31"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="27" t="s">
+      <c r="B23" s="28"/>
+      <c r="C23" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="26" t="s">
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="26"/>
-      <c r="C22" s="27" t="s">
+      <c r="B24" s="28"/>
+      <c r="C24" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A13:C13"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B11:C11"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="C2:F2"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="B10:C10"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
@@ -1621,22 +1731,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="14" t="s">

</xml_diff>

<commit_message>
POCOR-4148 - Update the default report card template with the competency period and item comments
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -1,19 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="27430"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
     <workbookView xWindow="13660" yWindow="900" windowWidth="22820" windowHeight="16060" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="24" r:id="rId1"/>
-    <sheet name="Competencies" sheetId="16" r:id="rId2"/>
-    <sheet name="Assessments" sheetId="18" r:id="rId3"/>
+    <sheet name="Competency Period Comments" sheetId="26" r:id="rId2"/>
+    <sheet name="Competency Item Comments" sheetId="25" r:id="rId3"/>
+    <sheet name="Competency Results" sheetId="16" r:id="rId4"/>
+    <sheet name="Assessments" sheetId="18" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">Assessments!$A$1:$E$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">Competencies!$A$1:$E$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">Assessments!$A$1:$E$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Competency Item Comments'!$A$1:$D$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Competency Period Comments'!$A$1:$C$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Competency Results'!$A$1:$E$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">General!$A$1:$G$25</definedName>
   </definedNames>
   <calcPr calcId="140000" concurrentCalc="0"/>
@@ -26,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="82">
   <si>
     <t>${InstitutionClasses.name}</t>
   </si>
@@ -70,9 +74,6 @@
     <t>Institution:</t>
   </si>
   <si>
-    <t>Competencies</t>
-  </si>
-  <si>
     <t>Template</t>
   </si>
   <si>
@@ -254,6 +255,27 @@
   </si>
   <si>
     <t>${InstitutionStudentsReportCards.body_mass.weight} kg</t>
+  </si>
+  <si>
+    <t>Competency Period Comments</t>
+  </si>
+  <si>
+    <t>Competency Item Comments</t>
+  </si>
+  <si>
+    <t>${"repeatRows":{"displayValue":"CompetencyTemplates.name","children":{"repeatRows":{"displayValue":"CompetencyPeriods.name","filter":"competency_template_id"}}}}</t>
+  </si>
+  <si>
+    <t>${"repeatRows":{"displayValue":"CompetencyTemplates.name","children":{"repeatRows":{"displayValue":"CompetencyPeriods.name","filter":"competency_template_id","children":{"repeatRows":{"displayValue":"CompetencyItems.name","filter":"competency_period_id"}}}}}}</t>
+  </si>
+  <si>
+    <t>${"match":{"displayValue":"StudentCompetencyPeriodComments.comments","rows":{"matchFrom":"CompetencyPeriods.id","matchTo":"StudentCompetencyPeriodComments.competency_period_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match":{"displayValue":"StudentCompetencyItemComments.comments","rows":{"matchFrom":"CompetencyPeriods.id","matchTo":"StudentCompetencyItemComments.competency_period_id","children":{"rows":{"matchFrom":"CompetencyItems.id","matchTo":"StudentCompetencyItemComments.competency_item_id","filter":"competency_period_id"}}}}}</t>
+  </si>
+  <si>
+    <t>Competency Results</t>
   </si>
 </sst>
 </file>
@@ -418,8 +440,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="181">
+  <cellStyleXfs count="185">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -674,42 +700,42 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -717,7 +743,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="181">
+  <cellStyles count="185">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -808,6 +834,8 @@
     <cellStyle name="Followed Hyperlink" xfId="176" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="178" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="180" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="182" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="184" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -898,6 +926,8 @@
     <cellStyle name="Hyperlink" xfId="175" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="177" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="179" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="181" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="183" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1285,7 +1315,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="27"/>
+      <c r="A1" s="32"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
       <c r="D1" s="1"/>
@@ -1294,18 +1324,18 @@
       <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:7" ht="26" customHeight="1">
-      <c r="A2" s="27"/>
+      <c r="A2" s="32"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="36" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
+      <c r="C2" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" ht="23" customHeight="1">
-      <c r="A3" s="27"/>
+      <c r="A3" s="32"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1326,32 +1356,32 @@
       <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="35"/>
+      <c r="C5" s="36"/>
       <c r="D5" s="20" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F5" s="22"/>
       <c r="G5" s="23"/>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="B6" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="35"/>
+        <v>65</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="36"/>
       <c r="D6" s="20" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F6" s="22"/>
       <c r="G6" s="23"/>
@@ -1360,15 +1390,15 @@
       <c r="A7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="34"/>
+      <c r="C7" s="35"/>
       <c r="D7" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="25" t="s">
         <v>68</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>69</v>
       </c>
       <c r="F7" s="22"/>
       <c r="G7" s="23"/>
@@ -1377,15 +1407,15 @@
       <c r="A8" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="34"/>
+      <c r="C8" s="35"/>
       <c r="D8" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F8" s="22"/>
       <c r="G8" s="23"/>
@@ -1394,15 +1424,15 @@
       <c r="A9" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="26"/>
+      <c r="C9" s="35"/>
       <c r="D9" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F9" s="22"/>
       <c r="G9" s="23"/>
@@ -1411,15 +1441,15 @@
       <c r="A10" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="35"/>
+      <c r="B10" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="36"/>
       <c r="D10" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F10" s="22"/>
       <c r="G10" s="23"/>
@@ -1428,15 +1458,15 @@
       <c r="A11" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="35"/>
+      <c r="C11" s="36"/>
       <c r="D11" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" s="25" t="s">
         <v>72</v>
-      </c>
-      <c r="E11" s="25" t="s">
-        <v>73</v>
       </c>
       <c r="F11" s="22"/>
       <c r="G11" s="23"/>
@@ -1451,23 +1481,23 @@
       <c r="G12" s="6"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
+      <c r="A13" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="33"/>
+      <c r="C13" s="33"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="27"/>
+      <c r="C14" s="8" t="s">
         <v>21</v>
-      </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="8" t="s">
-        <v>22</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
@@ -1475,12 +1505,12 @@
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="27"/>
+      <c r="C15" s="8" t="s">
         <v>23</v>
-      </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="8" t="s">
-        <v>24</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
@@ -1488,12 +1518,12 @@
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="27"/>
+      <c r="C16" s="8" t="s">
         <v>25</v>
-      </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="8" t="s">
-        <v>26</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
@@ -1511,7 +1541,7 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="30"/>
       <c r="C18" s="30"/>
@@ -1522,48 +1552,48 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="C19" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="E19" s="11" t="s">
+      <c r="F19" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="G19" s="11" t="s">
         <v>36</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="C20" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="D20" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="E20" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="E20" s="17" t="s">
-        <v>42</v>
-      </c>
       <c r="F20" s="21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="16" customHeight="1">
@@ -1577,7 +1607,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="29" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="30"/>
@@ -1587,38 +1617,33 @@
       <c r="G22" s="31"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="27"/>
+      <c r="C23" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="37" t="s">
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="37"/>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" s="28" t="s">
+      <c r="B24" s="27"/>
+      <c r="C24" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="28"/>
-      <c r="C24" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="A22:G22"/>
+  <mergeCells count="19">
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
@@ -1632,6 +1657,12 @@
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="A22:G22"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
@@ -1647,52 +1678,175 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="1" max="1" width="21.33203125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="69.6640625" style="4" customWidth="1"/>
+    <col min="4" max="16384" width="10.83203125" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967294" verticalDpi="4294967294"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="1" OnePage="0" WScale="100"/>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="1" max="1" width="17.5" style="4" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="30.33203125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="47" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967294" verticalDpi="4294967294"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="1" OnePage="0" WScale="100"/>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="17.5" style="4" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="29" style="4" customWidth="1"/>
-    <col min="4" max="4" width="34.33203125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="37.83203125" style="4" customWidth="1"/>
     <col min="5" max="5" width="16" style="4" customWidth="1"/>
     <col min="6" max="16384" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="32" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="A1" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="C2" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>18</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
       <c r="E3" s="17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1717,7 +1871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0"/>
@@ -1732,7 +1886,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="38" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B1" s="38"/>
       <c r="C1" s="38"/>
@@ -1741,7 +1895,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="39" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2" s="39"/>
       <c r="C2" s="39"/>
@@ -1750,36 +1904,36 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
POCOR-4156 - Update name to StudentBodyMassesController and UserBodyMassesTable. - UserBodyMassesTable under User plugin. - Update db name to user_body_masses. - Update healthBehavior. - Update NavigationComponent. - Update MessageTrait. - Update report_card_template.
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -247,13 +247,13 @@
     <t>BMI:</t>
   </si>
   <si>
-    <t>${InstitutionStudentsReportCards.body_mass.body_mass_index}</t>
-  </si>
-  <si>
-    <t>${InstitutionStudentsReportCards.body_mass.height} m</t>
-  </si>
-  <si>
-    <t>${InstitutionStudentsReportCards.body_mass.weight} kg</t>
+    <t>${InstitutionStudentsReportCards.student_body_mass.height} m</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.student_body_mass.weight} kg</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.student_body_mass.body_mass_index}</t>
   </si>
 </sst>
 </file>
@@ -677,21 +677,24 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -706,9 +709,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1285,7 +1285,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="27"/>
+      <c r="A1" s="32"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
       <c r="D1" s="1"/>
@@ -1294,18 +1294,18 @@
       <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:7" ht="26" customHeight="1">
-      <c r="A2" s="27"/>
+      <c r="A2" s="32"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="36" t="s">
+      <c r="C2" s="37" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" ht="23" customHeight="1">
-      <c r="A3" s="27"/>
+      <c r="A3" s="32"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1326,10 +1326,10 @@
       <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="35"/>
+      <c r="C5" s="36"/>
       <c r="D5" s="20" t="s">
         <v>11</v>
       </c>
@@ -1343,10 +1343,10 @@
       <c r="A6" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="35"/>
+      <c r="C6" s="36"/>
       <c r="D6" s="20" t="s">
         <v>10</v>
       </c>
@@ -1360,10 +1360,10 @@
       <c r="A7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="34"/>
+      <c r="C7" s="35"/>
       <c r="D7" s="20" t="s">
         <v>68</v>
       </c>
@@ -1377,10 +1377,10 @@
       <c r="A8" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="34"/>
+      <c r="C8" s="35"/>
       <c r="D8" s="20" t="s">
         <v>7</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>70</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F9" s="22"/>
       <c r="G9" s="23"/>
@@ -1411,15 +1411,15 @@
       <c r="A10" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="35"/>
+      <c r="C10" s="36"/>
       <c r="D10" s="20" t="s">
         <v>71</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F10" s="22"/>
       <c r="G10" s="23"/>
@@ -1428,15 +1428,15 @@
       <c r="A11" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="35"/>
+      <c r="C11" s="36"/>
       <c r="D11" s="20" t="s">
         <v>72</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F11" s="22"/>
       <c r="G11" s="23"/>
@@ -1451,21 +1451,21 @@
       <c r="G12" s="6"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
+      <c r="B13" s="33"/>
+      <c r="C13" s="33"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="28"/>
+      <c r="B14" s="27"/>
       <c r="C14" s="8" t="s">
         <v>22</v>
       </c>
@@ -1475,10 +1475,10 @@
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="27"/>
       <c r="C15" s="8" t="s">
         <v>24</v>
       </c>
@@ -1488,10 +1488,10 @@
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="28"/>
+      <c r="B16" s="27"/>
       <c r="C16" s="8" t="s">
         <v>26</v>
       </c>
@@ -1587,38 +1587,33 @@
       <c r="G22" s="31"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="37" t="s">
+      <c r="B23" s="27"/>
+      <c r="C23" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="37"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="28"/>
-      <c r="C24" s="37" t="s">
+      <c r="B24" s="27"/>
+      <c r="C24" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
@@ -1632,6 +1627,11 @@
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="A22:G22"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
@@ -1659,13 +1659,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="12" t="s">

</xml_diff>

<commit_message>
POCOR-4156 - Update the report_card_template.
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -247,13 +247,13 @@
     <t>BMI:</t>
   </si>
   <si>
-    <t>${InstitutionStudentsReportCards.student_body_mass.height} m</t>
-  </si>
-  <si>
-    <t>${InstitutionStudentsReportCards.student_body_mass.weight} kg</t>
-  </si>
-  <si>
-    <t>${InstitutionStudentsReportCards.student_body_mass.body_mass_index}</t>
+    <t>${InstitutionStudentsReportCards.student.body_mass_index}</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.student.weight} kg</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.student.height} m</t>
   </si>
 </sst>
 </file>
@@ -677,38 +677,38 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1285,7 +1285,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="32"/>
+      <c r="A1" s="27"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
       <c r="D1" s="1"/>
@@ -1294,18 +1294,18 @@
       <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:7" ht="26" customHeight="1">
-      <c r="A2" s="32"/>
+      <c r="A2" s="27"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" ht="23" customHeight="1">
-      <c r="A3" s="32"/>
+      <c r="A3" s="27"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1326,10 +1326,10 @@
       <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="36"/>
+      <c r="C5" s="35"/>
       <c r="D5" s="20" t="s">
         <v>11</v>
       </c>
@@ -1343,10 +1343,10 @@
       <c r="A6" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="36"/>
+      <c r="C6" s="35"/>
       <c r="D6" s="20" t="s">
         <v>10</v>
       </c>
@@ -1360,10 +1360,10 @@
       <c r="A7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="35"/>
+      <c r="C7" s="34"/>
       <c r="D7" s="20" t="s">
         <v>68</v>
       </c>
@@ -1377,10 +1377,10 @@
       <c r="A8" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="35"/>
+      <c r="C8" s="34"/>
       <c r="D8" s="20" t="s">
         <v>7</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>70</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F9" s="22"/>
       <c r="G9" s="23"/>
@@ -1411,10 +1411,10 @@
       <c r="A10" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="36"/>
+      <c r="C10" s="35"/>
       <c r="D10" s="20" t="s">
         <v>71</v>
       </c>
@@ -1428,15 +1428,15 @@
       <c r="A11" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="36"/>
+      <c r="C11" s="35"/>
       <c r="D11" s="20" t="s">
         <v>72</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F11" s="22"/>
       <c r="G11" s="23"/>
@@ -1451,21 +1451,21 @@
       <c r="G12" s="6"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="33"/>
-      <c r="C13" s="33"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="32"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="27"/>
+      <c r="B14" s="28"/>
       <c r="C14" s="8" t="s">
         <v>22</v>
       </c>
@@ -1475,10 +1475,10 @@
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="27"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="8" t="s">
         <v>24</v>
       </c>
@@ -1488,10 +1488,10 @@
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="27"/>
+      <c r="B16" s="28"/>
       <c r="C16" s="8" t="s">
         <v>26</v>
       </c>
@@ -1587,33 +1587,38 @@
       <c r="G22" s="31"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="27" t="s">
+      <c r="A23" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="28" t="s">
+      <c r="B23" s="28"/>
+      <c r="C23" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="28" t="s">
+      <c r="B24" s="28"/>
+      <c r="C24" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
@@ -1627,11 +1632,6 @@
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="A22:G22"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
@@ -1659,13 +1659,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="12" t="s">

</xml_diff>

<commit_message>
POCOR-4148 - Update report card template for bmi
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -248,15 +248,6 @@
     <t>BMI:</t>
   </si>
   <si>
-    <t>${InstitutionStudentsReportCards.body_mass.body_mass_index}</t>
-  </si>
-  <si>
-    <t>${InstitutionStudentsReportCards.body_mass.height} m</t>
-  </si>
-  <si>
-    <t>${InstitutionStudentsReportCards.body_mass.weight} kg</t>
-  </si>
-  <si>
     <t>Competency Period Comments</t>
   </si>
   <si>
@@ -276,6 +267,15 @@
   </si>
   <si>
     <t>Competency Results</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.student.height} m</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.student.weight} kg</t>
+  </si>
+  <si>
+    <t>${InstitutionStudentsReportCards.student.body_mass_index}</t>
   </si>
 </sst>
 </file>
@@ -703,38 +703,38 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1315,7 +1315,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="32"/>
+      <c r="A1" s="27"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
       <c r="D1" s="1"/>
@@ -1324,18 +1324,18 @@
       <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:7" ht="26" customHeight="1">
-      <c r="A2" s="32"/>
+      <c r="A2" s="27"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" ht="23" customHeight="1">
-      <c r="A3" s="32"/>
+      <c r="A3" s="27"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1356,10 +1356,10 @@
       <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="36"/>
+      <c r="C5" s="35"/>
       <c r="D5" s="20" t="s">
         <v>11</v>
       </c>
@@ -1373,10 +1373,10 @@
       <c r="A6" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="36"/>
+      <c r="C6" s="35"/>
       <c r="D6" s="20" t="s">
         <v>10</v>
       </c>
@@ -1390,10 +1390,10 @@
       <c r="A7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="35"/>
+      <c r="C7" s="34"/>
       <c r="D7" s="20" t="s">
         <v>67</v>
       </c>
@@ -1407,10 +1407,10 @@
       <c r="A8" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="35"/>
+      <c r="C8" s="34"/>
       <c r="D8" s="20" t="s">
         <v>7</v>
       </c>
@@ -1424,15 +1424,15 @@
       <c r="A9" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="35"/>
+      <c r="C9" s="34"/>
       <c r="D9" s="20" t="s">
         <v>69</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="F9" s="22"/>
       <c r="G9" s="23"/>
@@ -1441,15 +1441,15 @@
       <c r="A10" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="36"/>
+      <c r="C10" s="35"/>
       <c r="D10" s="20" t="s">
         <v>70</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F10" s="22"/>
       <c r="G10" s="23"/>
@@ -1458,15 +1458,15 @@
       <c r="A11" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="36"/>
+      <c r="C11" s="35"/>
       <c r="D11" s="20" t="s">
         <v>71</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="F11" s="22"/>
       <c r="G11" s="23"/>
@@ -1481,21 +1481,21 @@
       <c r="G12" s="6"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="33"/>
-      <c r="C13" s="33"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="32"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="27"/>
+      <c r="B14" s="28"/>
       <c r="C14" s="8" t="s">
         <v>21</v>
       </c>
@@ -1505,10 +1505,10 @@
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="27"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="8" t="s">
         <v>23</v>
       </c>
@@ -1518,10 +1518,10 @@
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="27"/>
+      <c r="B16" s="28"/>
       <c r="C16" s="8" t="s">
         <v>25</v>
       </c>
@@ -1617,33 +1617,38 @@
       <c r="G22" s="31"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="27" t="s">
+      <c r="A23" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="28" t="s">
+      <c r="B23" s="28"/>
+      <c r="C23" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="28" t="s">
+      <c r="B24" s="28"/>
+      <c r="C24" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
@@ -1658,11 +1663,6 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B9:C9"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="A22:G22"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
@@ -1688,11 +1688,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
+      <c r="A1" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="26" t="s">
@@ -1707,11 +1707,11 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="17" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1747,12 +1747,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="A1" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="26" t="s">
@@ -1770,12 +1770,12 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="17" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
       <c r="D3" s="17" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1813,13 +1813,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="33" t="s">
-        <v>81</v>
-      </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
+      <c r="A1" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="12" t="s">

</xml_diff>

<commit_message>
3.10.10 - Updated default template
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="21405"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
     <workbookView xWindow="13660" yWindow="900" windowWidth="22820" windowHeight="16060" tabRatio="500"/>
@@ -20,7 +20,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Competency Results'!$A$1:$E$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">General!$A$1:$G$25</definedName>
   </definedNames>
-  <calcPr calcId="140000" concurrentCalc="0"/>
+  <calcPr calcId="140000" iterateDelta="1E-4" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="83">
   <si>
     <t>${InstitutionClasses.name}</t>
   </si>
@@ -276,6 +276,10 @@
   </si>
   <si>
     <t>${InstitutionStudentsReportCards.student.body_mass_index}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${"image":{"displayValue":"Institutions.logo_content","imageWidth":"100","imageMarginLeft":"20","imageMarginTop":"5"}}
+</t>
   </si>
 </sst>
 </file>
@@ -627,7 +631,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -703,21 +707,24 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -733,14 +740,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="185">
@@ -933,49 +940,6 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>270932</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1041399</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>267547</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="270932" y="25400"/>
-          <a:ext cx="770467" cy="770467"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1315,7 +1279,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="27"/>
+      <c r="A1" s="40" t="s">
+        <v>82</v>
+      </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
       <c r="D1" s="1"/>
@@ -1324,18 +1290,18 @@
       <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:7" ht="26" customHeight="1">
-      <c r="A2" s="27"/>
+      <c r="A2" s="32"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="36" t="s">
+      <c r="C2" s="37" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" ht="23" customHeight="1">
-      <c r="A3" s="27"/>
+      <c r="A3" s="32"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1356,10 +1322,10 @@
       <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="35"/>
+      <c r="C5" s="36"/>
       <c r="D5" s="20" t="s">
         <v>11</v>
       </c>
@@ -1373,10 +1339,10 @@
       <c r="A6" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="35"/>
+      <c r="C6" s="36"/>
       <c r="D6" s="20" t="s">
         <v>10</v>
       </c>
@@ -1390,10 +1356,10 @@
       <c r="A7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="34"/>
+      <c r="C7" s="35"/>
       <c r="D7" s="20" t="s">
         <v>67</v>
       </c>
@@ -1407,10 +1373,10 @@
       <c r="A8" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="34"/>
+      <c r="C8" s="35"/>
       <c r="D8" s="20" t="s">
         <v>7</v>
       </c>
@@ -1424,10 +1390,10 @@
       <c r="A9" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="34"/>
+      <c r="C9" s="35"/>
       <c r="D9" s="20" t="s">
         <v>69</v>
       </c>
@@ -1441,10 +1407,10 @@
       <c r="A10" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="35"/>
+      <c r="C10" s="36"/>
       <c r="D10" s="20" t="s">
         <v>70</v>
       </c>
@@ -1458,10 +1424,10 @@
       <c r="A11" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="35"/>
+      <c r="C11" s="36"/>
       <c r="D11" s="20" t="s">
         <v>71</v>
       </c>
@@ -1481,21 +1447,21 @@
       <c r="G12" s="6"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
+      <c r="B13" s="33"/>
+      <c r="C13" s="33"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="28"/>
+      <c r="B14" s="27"/>
       <c r="C14" s="8" t="s">
         <v>21</v>
       </c>
@@ -1505,10 +1471,10 @@
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="27"/>
       <c r="C15" s="8" t="s">
         <v>23</v>
       </c>
@@ -1518,10 +1484,10 @@
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="28"/>
+      <c r="B16" s="27"/>
       <c r="C16" s="8" t="s">
         <v>25</v>
       </c>
@@ -1617,38 +1583,33 @@
       <c r="G22" s="31"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="37" t="s">
+      <c r="B23" s="27"/>
+      <c r="C23" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="37"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="28"/>
-      <c r="C24" s="37" t="s">
+      <c r="B24" s="27"/>
+      <c r="C24" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
@@ -1663,11 +1624,15 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B9:C9"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="A22:G22"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967294" verticalDpi="4294967294"/>
-  <drawing r:id="rId1"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
       <mx:PLV Mode="1" OnePage="0" WScale="100"/>
@@ -1688,11 +1653,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="26" t="s">
@@ -1747,12 +1712,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="26" t="s">
@@ -1813,13 +1778,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="12" t="s">

</xml_diff>

<commit_message>
POCOR- Include learning outcome into report card . Make changes to report_card.template to add placeholder for learning outcome(Outcome Subject Comment & Outcome Result)
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="21405"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="27430"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="13660" yWindow="900" windowWidth="22820" windowHeight="16060" tabRatio="500"/>
+    <workbookView xWindow="12760" yWindow="2560" windowWidth="22820" windowHeight="16060" tabRatio="500" firstSheet="3" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="24" r:id="rId1"/>
@@ -12,6 +12,8 @@
     <sheet name="Competency Item Comments" sheetId="25" r:id="rId3"/>
     <sheet name="Competency Results" sheetId="16" r:id="rId4"/>
     <sheet name="Assessments" sheetId="18" r:id="rId5"/>
+    <sheet name="Outcome Subject Comments" sheetId="27" r:id="rId6"/>
+    <sheet name="Outcome Result" sheetId="28" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="4">Assessments!$A$1:$E$5</definedName>
@@ -19,6 +21,8 @@
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Competency Period Comments'!$A$1:$C$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Competency Results'!$A$1:$E$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">General!$A$1:$G$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Outcome Result'!$A$1:$E$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Outcome Subject Comments'!$A$1:$D$4</definedName>
   </definedNames>
   <calcPr calcId="140000" iterateDelta="1E-4" concurrentCalc="0"/>
   <extLst>
@@ -30,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="89">
   <si>
     <t>${InstitutionClasses.name}</t>
   </si>
@@ -180,9 +184,6 @@
   </si>
   <si>
     <t xml:space="preserve">Assessments </t>
-  </si>
-  <si>
-    <t>${"match": {"displayValue": "StudentCompetencyResults.competency_grading_option.name","rows": {"matchFrom": "CompetencyPeriods.id","matchTo": "StudentCompetencyResults.competency_period_id","children": {"rows": {"matchFrom": "CompetencyCriterias.id","matchTo": "StudentCompetencyResults.competency_criteria_id","filter":"competency_period_id"}}}}}</t>
   </si>
   <si>
     <t>${InstitutionStudentsReportCards.student.name}</t>
@@ -280,6 +281,27 @@
   <si>
     <t xml:space="preserve">${"image":{"displayValue":"Institutions.logo_content","imageWidth":"100","imageMarginLeft":"20","imageMarginTop":"5"}}
 </t>
+  </si>
+  <si>
+    <t>Outcome Subject Comments</t>
+  </si>
+  <si>
+    <t>Subject</t>
+  </si>
+  <si>
+    <t>${"repeatRows":{"displayValue":"OutcomeTemplates.name","children":{"repeatRows":{"displayValue":"OutcomePeriods.name","filter":"outcome_template_id","children":{"repeatRows":{"displayValue":"OutcomeSubjects.name","filter":"outcome_period_id"}}}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${"repeatRows":{"displayValue":"OutcomeTemplates.name","children":{"repeatRows":{"displayValue":"OutcomePeriods.name","filter":"outcome_template_id", "children":{"repeatRows":{"displayValue":"OutcomeSubjects.name", "filter":"outcome_period_id", "children":{"repeatRows":{"displayValue":"OutcomeCriterias.name","filter":"outcome_subject_id"}}}}}}}}  </t>
+  </si>
+  <si>
+    <t>${"match":{"displayValue":"StudentOutcomeResults.outcome_grading_option.name","rows":{"matchFrom":"OutcomeTemplates.id","matchTo":"StudentOutcomeResults.outcome_template_id","children":{"rows":{"matchFrom":"OutcomePeriods.id","matchTo":"StudentOutcomeResults.outcome_period_id","filter":"outcome_template_id","children":{"rows":{"matchFrom":"OutcomeSubjects.education_subject_id","matchTo":"StudentOutcomeResults.education_subject_id","filter":"outcome_period_id","children":{"rows":{"matchFrom":"OutcomeCriterias.id","matchTo":"StudentOutcomeResults.outcome_criteria_id","filter":"outcome_subject_id"}}}}}}}}}</t>
+  </si>
+  <si>
+    <t>${"match":{"displayValue":"StudentOutcomeSubjectComments.comments","rows":{"matchFrom":"OutcomeTemplates.id","matchTo":"StudentOutcomeSubjectComments.outcome_template_id","children":{"rows":{"matchFrom":"OutcomePeriods.id","matchTo":"StudentOutcomeSubjectComments.outcome_period_id","filter":"outcome_template_id","children":{"rows":{"matchFrom":"OutcomeSubjects.education_subject_id","matchTo":"StudentOutcomeSubjectComments.education_subject_id","filter":"outcome_period_id"}}}}}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "StudentCompetencyResults.competency_grading_option.name","rows": {"matchFrom": "CompetencyPeriods.id","matchTo": "StudentCompetencyResults.competency_period_id","children": {"rows": {"matchFrom": "CompetencyCriterias.id","matchTo": "StudentCompetencyResults.competency_criteria_id","filter":"competency_period_id"}}}}}</t>
   </si>
 </sst>
 </file>
@@ -631,7 +653,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -707,6 +729,9 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -723,6 +748,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -745,9 +773,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="185">
@@ -1279,8 +1304,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="40" t="s">
-        <v>82</v>
+      <c r="A1" s="33" t="s">
+        <v>81</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
@@ -1290,18 +1315,18 @@
       <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:7" ht="26" customHeight="1">
-      <c r="A2" s="32"/>
+      <c r="A2" s="34"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="37" t="s">
-        <v>57</v>
-      </c>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="C2" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" ht="23" customHeight="1">
-      <c r="A3" s="32"/>
+      <c r="A3" s="34"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1322,32 +1347,32 @@
       <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="36"/>
+      <c r="C5" s="38"/>
       <c r="D5" s="20" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F5" s="22"/>
       <c r="G5" s="23"/>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="36" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" s="36"/>
+        <v>64</v>
+      </c>
+      <c r="B6" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="38"/>
       <c r="D6" s="20" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F6" s="22"/>
       <c r="G6" s="23"/>
@@ -1356,15 +1381,15 @@
       <c r="A7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="35"/>
+      <c r="C7" s="37"/>
       <c r="D7" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="25" t="s">
         <v>67</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>68</v>
       </c>
       <c r="F7" s="22"/>
       <c r="G7" s="23"/>
@@ -1373,15 +1398,15 @@
       <c r="A8" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="35"/>
+      <c r="C8" s="37"/>
       <c r="D8" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F8" s="22"/>
       <c r="G8" s="23"/>
@@ -1390,15 +1415,15 @@
       <c r="A9" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="35"/>
+      <c r="C9" s="37"/>
       <c r="D9" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F9" s="22"/>
       <c r="G9" s="23"/>
@@ -1407,15 +1432,15 @@
       <c r="A10" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="36" t="s">
-        <v>54</v>
-      </c>
-      <c r="C10" s="36"/>
+      <c r="B10" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="38"/>
       <c r="D10" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F10" s="22"/>
       <c r="G10" s="23"/>
@@ -1424,15 +1449,15 @@
       <c r="A11" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="36"/>
+      <c r="C11" s="38"/>
       <c r="D11" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F11" s="22"/>
       <c r="G11" s="23"/>
@@ -1447,21 +1472,21 @@
       <c r="G12" s="6"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="33"/>
-      <c r="C13" s="33"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="27"/>
+      <c r="B14" s="28"/>
       <c r="C14" s="8" t="s">
         <v>21</v>
       </c>
@@ -1471,10 +1496,10 @@
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="27"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="8" t="s">
         <v>23</v>
       </c>
@@ -1484,10 +1509,10 @@
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="27"/>
+      <c r="B16" s="28"/>
       <c r="C16" s="8" t="s">
         <v>25</v>
       </c>
@@ -1506,15 +1531,15 @@
       <c r="G17" s="10"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="29" t="s">
+      <c r="A18" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="31"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="32"/>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="11" t="s">
@@ -1524,10 +1549,10 @@
         <v>33</v>
       </c>
       <c r="C19" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="11" t="s">
         <v>59</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>60</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>34</v>
@@ -1556,10 +1581,10 @@
         <v>41</v>
       </c>
       <c r="F20" s="21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="16" customHeight="1">
@@ -1572,41 +1597,41 @@
       <c r="G21" s="6"/>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="31"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="32"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="27" t="s">
+      <c r="A23" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="28" t="s">
+      <c r="B23" s="28"/>
+      <c r="C23" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="28" t="s">
+      <c r="B24" s="28"/>
+      <c r="C24" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -1653,11 +1678,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="33" t="s">
-        <v>72</v>
-      </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
+      <c r="A1" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="26" t="s">
@@ -1672,11 +1697,11 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1712,12 +1737,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="33" t="s">
-        <v>73</v>
-      </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="A1" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="26" t="s">
@@ -1735,12 +1760,12 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
       <c r="D3" s="17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1778,13 +1803,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
+      <c r="A1" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="12" t="s">
@@ -1805,13 +1830,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
       <c r="E3" s="17" t="s">
-        <v>50</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1850,22 +1875,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="14" t="s">
@@ -1875,7 +1900,7 @@
         <v>46</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>45</v>
@@ -1889,13 +1914,13 @@
         <v>43</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E4" s="16" t="s">
         <v>42</v>
@@ -1915,4 +1940,141 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="1" max="1" width="17.5" style="4" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="30.33203125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="47" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="35" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967294" verticalDpi="4294967294"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="1" OnePage="0" WScale="100"/>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="1" max="1" width="17.5" style="4" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="37.83203125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="16" style="4" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967294" verticalDpi="4294967294"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="1" OnePage="0" WScale="100"/>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
POCOR-4508 - Added placeholders for subject comments in Outcome Results tab in the default report card template.
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
   <workbookPr autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="6480" yWindow="2140" windowWidth="25600" windowHeight="15620" tabRatio="500" firstSheet="2" activeTab="3"/>
+    <workbookView xWindow="6480" yWindow="2140" windowWidth="25600" windowHeight="15620" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Competency Results" sheetId="4" r:id="rId4"/>
     <sheet name="Assessments" sheetId="5" r:id="rId5"/>
     <sheet name="Outcome Subject Comments" sheetId="6" r:id="rId6"/>
-    <sheet name="Outcome Result" sheetId="7" r:id="rId7"/>
+    <sheet name="Outcome Results" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="140001" concurrentCalc="0"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="108">
   <si>
     <t>Competency Item Comments</t>
   </si>
@@ -345,6 +345,12 @@
   <si>
     <t>${"match":{"displayValue":"StudentCompetencyItemComments.comments","rows":{"matchFrom":"CompetencyTemplates.id","matchTo":"StudentCompetencyItemComments.competency_template_id","children":{"rows":{"matchFrom":"CompetencyPeriods.id","matchTo":"StudentCompetencyItemComments.competency_period_id","filter":"competency_template_id","children":{"rows":{"matchFrom":"CompetencyItems.id","matchTo":"StudentCompetencyItemComments.competency_item_id","filter":"competency_period_id","mergeBy":{"mergeFrom":"CompetencyCriterias.id","filter":"competency_item_id"}}}}}}}}</t>
   </si>
+  <si>
+    <t>Subject Comments</t>
+  </si>
+  <si>
+    <t>${"match":{"displayValue":"StudentOutcomeSubjectComments.comments","rows":{"matchFrom":"OutcomeTemplates.id","matchTo":"StudentOutcomeSubjectComments.outcome_template_id","children":{"rows":{"matchFrom":"OutcomePeriods.id","matchTo":"StudentOutcomeSubjectComments.outcome_period_id","filter":"outcome_template_id","children":{"rows":{"matchFrom":"OutcomeSubjects.education_subject_id","matchTo":"StudentOutcomeSubjectComments.education_subject_id","filter":"outcome_period_id","mergeBy":{"mergeFrom":"OutcomeCriterias.id","filter":"outcome_subject_id"}}}}}}}}</t>
+  </si>
 </sst>
 </file>
 
@@ -419,7 +425,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -540,13 +546,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -610,25 +633,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -636,8 +651,19 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -645,16 +671,18 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="5">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -998,7 +1026,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="32" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1"/>
@@ -1019,14 +1047,14 @@
       <c r="Q1" s="3"/>
     </row>
     <row r="2" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A2" s="37"/>
+      <c r="A2" s="33"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
       <c r="G2" s="6"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
@@ -1040,7 +1068,7 @@
       <c r="Q2" s="3"/>
     </row>
     <row r="3" spans="1:17" ht="22.5" customHeight="1">
-      <c r="A3" s="37"/>
+      <c r="A3" s="33"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1081,10 +1109,10 @@
       <c r="A5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="28"/>
+      <c r="C5" s="31"/>
       <c r="D5" s="11" t="s">
         <v>14</v>
       </c>
@@ -1108,10 +1136,10 @@
       <c r="A6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="28"/>
+      <c r="C6" s="31"/>
       <c r="D6" s="11" t="s">
         <v>18</v>
       </c>
@@ -1135,10 +1163,10 @@
       <c r="A7" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="28"/>
+      <c r="C7" s="31"/>
       <c r="D7" s="11" t="s">
         <v>22</v>
       </c>
@@ -1162,10 +1190,10 @@
       <c r="A8" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="28"/>
+      <c r="C8" s="31"/>
       <c r="D8" s="11" t="s">
         <v>26</v>
       </c>
@@ -1189,10 +1217,10 @@
       <c r="A9" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="28"/>
+      <c r="C9" s="31"/>
       <c r="D9" s="11" t="s">
         <v>30</v>
       </c>
@@ -1216,10 +1244,10 @@
       <c r="A10" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="28"/>
+      <c r="C10" s="31"/>
       <c r="D10" s="11" t="s">
         <v>34</v>
       </c>
@@ -1243,10 +1271,10 @@
       <c r="A11" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="28"/>
+      <c r="C11" s="31"/>
       <c r="D11" s="11" t="s">
         <v>38</v>
       </c>
@@ -1270,10 +1298,10 @@
       <c r="A12" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="28"/>
+      <c r="C12" s="31"/>
       <c r="D12" s="11" t="s">
         <v>42</v>
       </c>
@@ -1297,10 +1325,10 @@
       <c r="A13" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="28"/>
+      <c r="C13" s="31"/>
       <c r="D13" s="17"/>
       <c r="E13" s="18"/>
       <c r="F13" s="13"/>
@@ -1320,10 +1348,10 @@
       <c r="A14" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="28"/>
+      <c r="C14" s="31"/>
       <c r="D14" s="17"/>
       <c r="E14" s="18"/>
       <c r="F14" s="13"/>
@@ -1359,11 +1387,11 @@
       <c r="Q15" s="3"/>
     </row>
     <row r="16" spans="1:17" ht="12" customHeight="1">
-      <c r="A16" s="35" t="s">
+      <c r="A16" s="38" t="s">
         <v>48</v>
       </c>
       <c r="B16" s="30"/>
-      <c r="C16" s="28"/>
+      <c r="C16" s="31"/>
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
       <c r="F16" s="20"/>
@@ -1380,10 +1408,10 @@
       <c r="Q16" s="3"/>
     </row>
     <row r="17" spans="1:17" ht="12" customHeight="1">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="34"/>
+      <c r="B17" s="37"/>
       <c r="C17" s="25" t="s">
         <v>59</v>
       </c>
@@ -1403,10 +1431,10 @@
       <c r="Q17" s="3"/>
     </row>
     <row r="18" spans="1:17" ht="12" customHeight="1">
-      <c r="A18" s="33" t="s">
+      <c r="A18" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="B18" s="34"/>
+      <c r="B18" s="37"/>
       <c r="C18" s="25" t="s">
         <v>70</v>
       </c>
@@ -1426,10 +1454,10 @@
       <c r="Q18" s="3"/>
     </row>
     <row r="19" spans="1:17" ht="12" customHeight="1">
-      <c r="A19" s="33" t="s">
+      <c r="A19" s="36" t="s">
         <v>71</v>
       </c>
-      <c r="B19" s="34"/>
+      <c r="B19" s="37"/>
       <c r="C19" s="25" t="s">
         <v>72</v>
       </c>
@@ -1449,10 +1477,10 @@
       <c r="Q19" s="3"/>
     </row>
     <row r="20" spans="1:17" ht="12" customHeight="1">
-      <c r="A20" s="33" t="s">
+      <c r="A20" s="36" t="s">
         <v>73</v>
       </c>
-      <c r="B20" s="34"/>
+      <c r="B20" s="37"/>
       <c r="C20" s="25" t="s">
         <v>74</v>
       </c>
@@ -1491,7 +1519,7 @@
       <c r="Q21" s="3"/>
     </row>
     <row r="22" spans="1:17" ht="12" customHeight="1">
-      <c r="A22" s="32" t="s">
+      <c r="A22" s="29" t="s">
         <v>75</v>
       </c>
       <c r="B22" s="30"/>
@@ -1499,7 +1527,7 @@
       <c r="D22" s="30"/>
       <c r="E22" s="30"/>
       <c r="F22" s="30"/>
-      <c r="G22" s="28"/>
+      <c r="G22" s="31"/>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
@@ -1597,7 +1625,7 @@
       <c r="Q25" s="3"/>
     </row>
     <row r="26" spans="1:17" ht="12" customHeight="1">
-      <c r="A26" s="32" t="s">
+      <c r="A26" s="29" t="s">
         <v>6</v>
       </c>
       <c r="B26" s="30"/>
@@ -1605,7 +1633,7 @@
       <c r="D26" s="30"/>
       <c r="E26" s="30"/>
       <c r="F26" s="30"/>
-      <c r="G26" s="28"/>
+      <c r="G26" s="31"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
@@ -1618,17 +1646,17 @@
       <c r="Q26" s="3"/>
     </row>
     <row r="27" spans="1:17" ht="12" customHeight="1">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="40" t="s">
         <v>90</v>
       </c>
-      <c r="B27" s="28"/>
-      <c r="C27" s="29" t="s">
+      <c r="B27" s="31"/>
+      <c r="C27" s="39" t="s">
         <v>91</v>
       </c>
       <c r="D27" s="30"/>
       <c r="E27" s="30"/>
       <c r="F27" s="30"/>
-      <c r="G27" s="28"/>
+      <c r="G27" s="31"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
@@ -1641,17 +1669,17 @@
       <c r="Q27" s="3"/>
     </row>
     <row r="28" spans="1:17" ht="12" customHeight="1">
-      <c r="A28" s="31" t="s">
+      <c r="A28" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29" t="s">
+      <c r="B28" s="31"/>
+      <c r="C28" s="39" t="s">
         <v>93</v>
       </c>
       <c r="D28" s="30"/>
       <c r="E28" s="30"/>
       <c r="F28" s="30"/>
-      <c r="G28" s="28"/>
+      <c r="G28" s="31"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
@@ -2655,6 +2683,13 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A26:G26"/>
     <mergeCell ref="A22:G22"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="C2:F2"/>
@@ -2667,17 +2702,10 @@
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A16:C16"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A26:G26"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
   </mergeCells>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -2702,11 +2730,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="12" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="29" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="30"/>
-      <c r="C1" s="28"/>
+      <c r="C1" s="31"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -4035,12 +4063,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
-      <c r="D1" s="28"/>
+      <c r="D1" s="31"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
@@ -5394,16 +5422,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
@@ -5458,10 +5486,10 @@
       <c r="F3" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="42" t="s">
+      <c r="G3" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="H3" s="43" t="s">
+      <c r="H3" s="28" t="s">
         <v>104</v>
       </c>
       <c r="I3" s="3"/>
@@ -6786,13 +6814,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="29" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
       <c r="D1" s="30"/>
-      <c r="E1" s="28"/>
+      <c r="E1" s="31"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
@@ -6805,13 +6833,13 @@
       <c r="O1" s="3"/>
     </row>
     <row r="2" spans="1:15" ht="12" customHeight="1">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>51</v>
       </c>
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
       <c r="D2" s="30"/>
-      <c r="E2" s="28"/>
+      <c r="E2" s="31"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -8174,12 +8202,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="29" t="s">
         <v>94</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
-      <c r="D1" s="28"/>
+      <c r="D1" s="31"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
@@ -9526,19 +9554,19 @@
     <col min="3" max="3" width="25.6640625" customWidth="1"/>
     <col min="4" max="4" width="37.83203125" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="23.83203125" customWidth="1"/>
     <col min="7" max="15" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
@@ -9565,7 +9593,9 @@
       <c r="E2" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="21" t="s">
+        <v>106</v>
+      </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
@@ -9586,7 +9616,9 @@
       <c r="E3" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="F3" s="3"/>
+      <c r="F3" s="44" t="s">
+        <v>107</v>
+      </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -10884,7 +10916,7 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
POCOR-4528 - Fixed placeholders for Comments in Competency Period Comments and Competency Item Comments
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
   <workbookPr autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="6480" yWindow="2140" windowWidth="25600" windowHeight="15620" tabRatio="500"/>
+    <workbookView xWindow="10640" yWindow="2480" windowWidth="25600" windowHeight="15620" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -55,9 +55,6 @@
     <t>Institution:</t>
   </si>
   <si>
-    <t>${"match":{"displayValue":"StudentCompetencyPeriodComments.comments","rows":{"matchFrom":"CompetencyPeriods.id","matchTo":"StudentCompetencyPeriodComments.competency_period_id"}}}</t>
-  </si>
-  <si>
     <t>${Institutions.code_name}</t>
   </si>
   <si>
@@ -65,9 +62,6 @@
   </si>
   <si>
     <t>${"repeatRows":{"displayValue":"CompetencyTemplates.name","children":{"repeatRows":{"displayValue":"CompetencyPeriods.name","filter":"competency_template_id","children":{"repeatRows":{"displayValue":"CompetencyItems.name","filter":"competency_period_id"}}}}}}</t>
-  </si>
-  <si>
-    <t>${"match":{"displayValue":"StudentCompetencyItemComments.comments","rows":{"matchFrom":"CompetencyPeriods.id","matchTo":"StudentCompetencyItemComments.competency_period_id","children":{"rows":{"matchFrom":"CompetencyItems.id","matchTo":"StudentCompetencyItemComments.competency_item_id","filter":"competency_period_id"}}}}}</t>
   </si>
   <si>
     <t>Student:</t>
@@ -351,6 +345,13 @@
   <si>
     <t>${"match":{"displayValue":"StudentOutcomeSubjectComments.comments","rows":{"matchFrom":"OutcomeTemplates.id","matchTo":"StudentOutcomeSubjectComments.outcome_template_id","children":{"rows":{"matchFrom":"OutcomePeriods.id","matchTo":"StudentOutcomeSubjectComments.outcome_period_id","filter":"outcome_template_id","children":{"rows":{"matchFrom":"OutcomeSubjects.education_subject_id","matchTo":"StudentOutcomeSubjectComments.education_subject_id","filter":"outcome_period_id","mergeBy":{"mergeFrom":"OutcomeCriterias.id","filter":"outcome_subject_id"}}}}}}}}</t>
   </si>
+  <si>
+    <t xml:space="preserve">${"match":{"displayValue":"StudentCompetencyPeriodComments.comments","rows":{"matchFrom":"CompetencyTemplates.id","matchTo":"StudentCompetencyPeriodComments.competency_template_id","children":{"rows":{"matchFrom":"CompetencyPeriods.id","matchTo":"StudentCompetencyPeriodComments.competency_period_id","filter":"competency_template_id"}}}}}
+</t>
+  </si>
+  <si>
+    <t>${"match":{"displayValue":"StudentCompetencyItemComments.comments","rows":{"matchFrom":"CompetencyTemplates.id","matchTo":"StudentCompetencyItemComments.competency_template_id","children":{"rows":{"matchFrom":"CompetencyPeriods.id","matchTo":"StudentCompetencyItemComments.competency_period_id","filter":"competency_template_id","children":{"rows":{"matchFrom":"CompetencyItems.id","matchTo":"StudentCompetencyItemComments.competency_item_id","filter":"competency_period_id"}}}}}}}</t>
+  </si>
 </sst>
 </file>
 
@@ -569,7 +570,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -639,11 +640,23 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -651,19 +664,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -674,8 +678,8 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1026,7 +1030,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="36" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1"/>
@@ -1047,14 +1051,14 @@
       <c r="Q1" s="3"/>
     </row>
     <row r="2" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A2" s="33"/>
+      <c r="A2" s="37"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="34" t="s">
+      <c r="C2" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="6"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
@@ -1068,7 +1072,7 @@
       <c r="Q2" s="3"/>
     </row>
     <row r="3" spans="1:17" ht="22.5" customHeight="1">
-      <c r="A3" s="33"/>
+      <c r="A3" s="37"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1109,15 +1113,15 @@
       <c r="A5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="35" t="s">
-        <v>10</v>
+      <c r="B5" s="30" t="s">
+        <v>9</v>
       </c>
       <c r="C5" s="31"/>
       <c r="D5" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F5" s="13"/>
       <c r="G5" s="3"/>
@@ -1134,17 +1138,17 @@
     </row>
     <row r="6" spans="1:17" ht="12" customHeight="1">
       <c r="A6" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="35" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>15</v>
       </c>
       <c r="C6" s="31"/>
       <c r="D6" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F6" s="13"/>
       <c r="G6" s="3"/>
@@ -1161,17 +1165,17 @@
     </row>
     <row r="7" spans="1:17" ht="12" customHeight="1">
       <c r="A7" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="35" t="s">
-        <v>21</v>
+        <v>18</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>19</v>
       </c>
       <c r="C7" s="31"/>
       <c r="D7" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F7" s="13"/>
       <c r="G7" s="3"/>
@@ -1188,17 +1192,17 @@
     </row>
     <row r="8" spans="1:17" ht="12" customHeight="1">
       <c r="A8" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="35" t="s">
-        <v>25</v>
+        <v>22</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="C8" s="31"/>
       <c r="D8" s="11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F8" s="13"/>
       <c r="G8" s="3"/>
@@ -1215,17 +1219,17 @@
     </row>
     <row r="9" spans="1:17" ht="12" customHeight="1">
       <c r="A9" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="35" t="s">
-        <v>29</v>
+        <v>26</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>27</v>
       </c>
       <c r="C9" s="31"/>
       <c r="D9" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F9" s="13"/>
       <c r="G9" s="3"/>
@@ -1242,17 +1246,17 @@
     </row>
     <row r="10" spans="1:17" ht="12" customHeight="1">
       <c r="A10" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="35" t="s">
-        <v>33</v>
+        <v>30</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>31</v>
       </c>
       <c r="C10" s="31"/>
       <c r="D10" s="11" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F10" s="13"/>
       <c r="G10" s="3"/>
@@ -1269,17 +1273,17 @@
     </row>
     <row r="11" spans="1:17" ht="12" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="35" t="s">
-        <v>37</v>
+        <v>34</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>35</v>
       </c>
       <c r="C11" s="31"/>
       <c r="D11" s="11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F11" s="13"/>
       <c r="G11" s="3"/>
@@ -1296,17 +1300,17 @@
     </row>
     <row r="12" spans="1:17" ht="12" customHeight="1">
       <c r="A12" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B12" s="35" t="s">
-        <v>41</v>
+        <v>38</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>39</v>
       </c>
       <c r="C12" s="31"/>
       <c r="D12" s="11" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="3"/>
@@ -1323,10 +1327,10 @@
     </row>
     <row r="13" spans="1:17" ht="12" customHeight="1">
       <c r="A13" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="35" t="s">
-        <v>45</v>
+        <v>42</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>43</v>
       </c>
       <c r="C13" s="31"/>
       <c r="D13" s="17"/>
@@ -1346,10 +1350,10 @@
     </row>
     <row r="14" spans="1:17" ht="12" customHeight="1">
       <c r="A14" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" s="35" t="s">
-        <v>47</v>
+        <v>44</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>45</v>
       </c>
       <c r="C14" s="31"/>
       <c r="D14" s="17"/>
@@ -1387,10 +1391,10 @@
       <c r="Q15" s="3"/>
     </row>
     <row r="16" spans="1:17" ht="12" customHeight="1">
-      <c r="A16" s="38" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" s="30"/>
+      <c r="A16" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="33"/>
       <c r="C16" s="31"/>
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
@@ -1408,12 +1412,12 @@
       <c r="Q16" s="3"/>
     </row>
     <row r="17" spans="1:17" ht="12" customHeight="1">
-      <c r="A17" s="36" t="s">
-        <v>54</v>
-      </c>
-      <c r="B17" s="37"/>
+      <c r="A17" s="39" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" s="40"/>
       <c r="C17" s="25" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D17" s="26"/>
       <c r="E17" s="26"/>
@@ -1431,12 +1435,12 @@
       <c r="Q17" s="3"/>
     </row>
     <row r="18" spans="1:17" ht="12" customHeight="1">
-      <c r="A18" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18" s="37"/>
+      <c r="A18" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="40"/>
       <c r="C18" s="25" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D18" s="26"/>
       <c r="E18" s="26"/>
@@ -1454,12 +1458,12 @@
       <c r="Q18" s="3"/>
     </row>
     <row r="19" spans="1:17" ht="12" customHeight="1">
-      <c r="A19" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="B19" s="37"/>
+      <c r="A19" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="B19" s="40"/>
       <c r="C19" s="25" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D19" s="26"/>
       <c r="E19" s="26"/>
@@ -1477,12 +1481,12 @@
       <c r="Q19" s="3"/>
     </row>
     <row r="20" spans="1:17" ht="12" customHeight="1">
-      <c r="A20" s="36" t="s">
-        <v>73</v>
-      </c>
-      <c r="B20" s="37"/>
+      <c r="A20" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="40"/>
       <c r="C20" s="25" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D20" s="26"/>
       <c r="E20" s="26"/>
@@ -1519,14 +1523,14 @@
       <c r="Q21" s="3"/>
     </row>
     <row r="22" spans="1:17" ht="12" customHeight="1">
-      <c r="A22" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
+      <c r="A22" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
       <c r="G22" s="31"/>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
@@ -1541,25 +1545,25 @@
     </row>
     <row r="23" spans="1:17" ht="12" customHeight="1">
       <c r="A23" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C23" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="D23" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="E23" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="D23" s="24" t="s">
+      <c r="F23" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="G23" s="24" t="s">
         <v>80</v>
-      </c>
-      <c r="F23" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="G23" s="24" t="s">
-        <v>82</v>
       </c>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
@@ -1574,25 +1578,25 @@
     </row>
     <row r="24" spans="1:17" ht="12" customHeight="1">
       <c r="A24" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="D24" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="E24" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="F24" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="G24" s="9" t="s">
         <v>87</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>89</v>
       </c>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
@@ -1625,14 +1629,14 @@
       <c r="Q25" s="3"/>
     </row>
     <row r="26" spans="1:17" ht="12" customHeight="1">
-      <c r="A26" s="29" t="s">
+      <c r="A26" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="B26" s="30"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="30"/>
+      <c r="B26" s="33"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
       <c r="G26" s="31"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
@@ -1646,16 +1650,16 @@
       <c r="Q26" s="3"/>
     </row>
     <row r="27" spans="1:17" ht="12" customHeight="1">
-      <c r="A27" s="40" t="s">
-        <v>90</v>
+      <c r="A27" s="34" t="s">
+        <v>88</v>
       </c>
       <c r="B27" s="31"/>
-      <c r="C27" s="39" t="s">
-        <v>91</v>
-      </c>
-      <c r="D27" s="30"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="30"/>
+      <c r="C27" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
       <c r="G27" s="31"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
@@ -1669,16 +1673,16 @@
       <c r="Q27" s="3"/>
     </row>
     <row r="28" spans="1:17" ht="12" customHeight="1">
-      <c r="A28" s="40" t="s">
-        <v>92</v>
+      <c r="A28" s="34" t="s">
+        <v>90</v>
       </c>
       <c r="B28" s="31"/>
-      <c r="C28" s="39" t="s">
-        <v>93</v>
-      </c>
-      <c r="D28" s="30"/>
-      <c r="E28" s="30"/>
-      <c r="F28" s="30"/>
+      <c r="C28" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
       <c r="G28" s="31"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
@@ -2683,6 +2687,16 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="C27:G27"/>
@@ -2691,21 +2705,11 @@
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B13:C13"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A16:C16"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B7:C7"/>
   </mergeCells>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75000000000000011" bottom="0.75000000000000011" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -2730,10 +2734,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="12" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="30"/>
+      <c r="B1" s="33"/>
       <c r="C1" s="31"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
@@ -2772,8 +2776,8 @@
         <v>7</v>
       </c>
       <c r="B3" s="9"/>
-      <c r="C3" s="9" t="s">
-        <v>9</v>
+      <c r="C3" s="45" t="s">
+        <v>106</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -4063,11 +4067,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="31"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -4088,7 +4092,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>6</v>
@@ -4106,12 +4110,12 @@
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9" t="s">
-        <v>13</v>
+        <v>107</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -5422,16 +5426,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="41" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
+      <c r="A1" s="42" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
@@ -5448,22 +5452,22 @@
         <v>5</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F2" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="G2" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="H2" s="21" t="s">
         <v>101</v>
-      </c>
-      <c r="G2" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="H2" s="21" t="s">
-        <v>103</v>
       </c>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
@@ -5475,22 +5479,22 @@
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
       <c r="E3" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G3" s="27" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H3" s="28" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -6814,12 +6818,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
+      <c r="A1" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
       <c r="E1" s="31"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
@@ -6833,12 +6837,12 @@
       <c r="O1" s="3"/>
     </row>
     <row r="2" spans="1:15" ht="12" customHeight="1">
-      <c r="A2" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
+      <c r="A2" s="44" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
       <c r="E2" s="31"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
@@ -6853,19 +6857,19 @@
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
       <c r="A3" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="C3" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="E3" s="24" t="s">
         <v>61</v>
-      </c>
-      <c r="D3" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="E3" s="24" t="s">
-        <v>63</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -6880,19 +6884,19 @@
     </row>
     <row r="4" spans="1:15" ht="12" customHeight="1">
       <c r="A4" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>66</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>68</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -8202,11 +8206,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="29" t="s">
-        <v>94</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="A1" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="31"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -8227,7 +8231,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>6</v>
@@ -8245,12 +8249,12 @@
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -9559,14 +9563,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="41" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
+      <c r="A1" s="42" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
@@ -9585,16 +9589,16 @@
         <v>5</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -9608,16 +9612,16 @@
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
       <c r="E3" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="F3" s="44" t="s">
-        <v>107</v>
+        <v>97</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>105</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>

</xml_diff>

<commit_message>
POCOR-5814:subject name showing in institution_subjects table|status:Done
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" state="visible" r:id="rId2"/>
@@ -349,7 +349,7 @@
     <t xml:space="preserve">Additional comments</t>
   </si>
   <si>
-    <t xml:space="preserve">${"repeatRows":{"displayValue":"AssessmentItems.education_subject.name"}}</t>
+    <t xml:space="preserve">${"repeatRows":{"displayValue":"InstitutionSubjectStudentsWithName.institution_subject.name"}}</t>
   </si>
   <si>
     <t xml:space="preserve">${"match": {"displayValue": "SubjectTeacher.name","rows": {"matchFrom": "SubjectTeacher.education_subject_id","matchTo": "SubjectTeacher.education_subject_id"}}}</t>
@@ -408,6 +408,7 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -429,6 +430,7 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -436,6 +438,7 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -443,6 +446,7 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -450,18 +454,21 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF2A3238"/>
       <name val="lato_regular"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -545,7 +552,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -565,7 +572,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -683,12 +690,12 @@
     </xf>
   </cellXfs>
   <cellStyles count="6">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -2585,276 +2592,24 @@
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
     </row>
-    <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-    </row>
-    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-    </row>
+    <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3840,7 +3595,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -3928,294 +3683,24 @@
       <c r="M3" s="5"/>
       <c r="N3" s="5"/>
     </row>
-    <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-    </row>
-    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-    </row>
+    <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -5201,7 +4686,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -5309,312 +4794,24 @@
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
     </row>
-    <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
-    </row>
-    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-    </row>
+    <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -6600,7 +5797,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -6727,312 +5924,23 @@
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
     </row>
-    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
-      <c r="P7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
-      <c r="P8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="5"/>
-      <c r="P9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
-      <c r="P11" s="5"/>
-    </row>
-    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
-      <c r="P12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="5"/>
-      <c r="P15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5"/>
-      <c r="P16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5"/>
-      <c r="P17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5"/>
-      <c r="P18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-      <c r="P20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-    </row>
+    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -8019,7 +6927,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -8107,294 +7015,24 @@
       <c r="M3" s="5"/>
       <c r="N3" s="5"/>
     </row>
-    <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-    </row>
-    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-    </row>
+    <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -9380,7 +8018,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -9478,312 +8116,24 @@
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
     </row>
-    <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
-    </row>
-    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-    </row>
+    <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -10769,7 +9119,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
POCOR:6810: code enhance for subject placeholder in assessment tab | Status: Done
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25225"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\poona\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0CC27BA-0563-4CC5-AA74-E8603F13D81E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10305" tabRatio="500" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -354,9 +348,6 @@
     <t>Additional comments</t>
   </si>
   <si>
-    <t>${"repeatRows":{"displayValue":"InstitutionSubjectStudentsWithName.institution_subject.name"}}</t>
-  </si>
-  <si>
     <t>Outcome Subject Comments</t>
   </si>
   <si>
@@ -397,12 +388,15 @@
   </si>
   <si>
     <t>${"match": {"displayValue": "InstitutionStudentsReportCardsComments.comments","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.education_subject_id","matchTo": "InstitutionSubjectStudentsWithName.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionSubjectStudentsWithName.name","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.id","matchTo": "InstitutionSubjectStudentsWithName.id"}}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="7">
     <font>
       <sz val="12"/>
@@ -524,7 +518,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -590,6 +584,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -597,25 +604,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -746,7 +743,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -778,27 +775,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -830,24 +809,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1023,24 +984,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q999"/>
-  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="16.58203125" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.625" customWidth="1"/>
+    <col min="2" max="2" width="14.375" customWidth="1"/>
     <col min="3" max="3" width="15.75" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.875" customWidth="1"/>
     <col min="5" max="5" width="27.75" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="10.5" customWidth="1"/>
-    <col min="8" max="17" width="10.33203125" customWidth="1"/>
+    <col min="8" max="17" width="10.375" customWidth="1"/>
     <col min="18" max="26" width="11" customWidth="1"/>
     <col min="27" max="1025" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" customHeight="1">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
@@ -1061,14 +1022,14 @@
       <c r="Q1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A2" s="31"/>
+      <c r="A2" s="25"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="32" t="s">
+      <c r="C2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
       <c r="G2" s="5"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -1082,7 +1043,7 @@
       <c r="Q2" s="4"/>
     </row>
     <row r="3" spans="1:17" ht="22.5" customHeight="1">
-      <c r="A3" s="31"/>
+      <c r="A3" s="25"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1123,10 +1084,10 @@
       <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="30"/>
+      <c r="C5" s="27"/>
       <c r="D5" s="8" t="s">
         <v>4</v>
       </c>
@@ -1150,10 +1111,10 @@
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="30"/>
+      <c r="C6" s="27"/>
       <c r="D6" s="8" t="s">
         <v>8</v>
       </c>
@@ -1177,10 +1138,10 @@
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="30"/>
+      <c r="C7" s="27"/>
       <c r="D7" s="12" t="s">
         <v>12</v>
       </c>
@@ -1204,10 +1165,10 @@
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="30"/>
+      <c r="C8" s="27"/>
       <c r="D8" s="12" t="s">
         <v>16</v>
       </c>
@@ -1231,10 +1192,10 @@
       <c r="A9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="30"/>
+      <c r="C9" s="27"/>
       <c r="D9" s="12" t="s">
         <v>20</v>
       </c>
@@ -1258,10 +1219,10 @@
       <c r="A10" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="30"/>
+      <c r="C10" s="27"/>
       <c r="D10" s="12" t="s">
         <v>24</v>
       </c>
@@ -1285,10 +1246,10 @@
       <c r="A11" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="30"/>
+      <c r="C11" s="27"/>
       <c r="D11" s="12" t="s">
         <v>28</v>
       </c>
@@ -1312,10 +1273,10 @@
       <c r="A12" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="30" t="s">
+      <c r="B12" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="30"/>
+      <c r="C12" s="27"/>
       <c r="D12" s="12" t="s">
         <v>32</v>
       </c>
@@ -1339,10 +1300,10 @@
       <c r="A13" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="30"/>
+      <c r="C13" s="27"/>
       <c r="D13" s="12" t="s">
         <v>36</v>
       </c>
@@ -1366,10 +1327,10 @@
       <c r="A14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="30" t="s">
+      <c r="B14" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="30"/>
+      <c r="C14" s="27"/>
       <c r="D14" s="12" t="s">
         <v>40</v>
       </c>
@@ -1409,11 +1370,11 @@
       <c r="Q15" s="4"/>
     </row>
     <row r="16" spans="1:17" ht="12" customHeight="1">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
       <c r="D16" s="15"/>
       <c r="E16" s="15"/>
       <c r="F16" s="15"/>
@@ -1430,10 +1391,10 @@
       <c r="Q16" s="4"/>
     </row>
     <row r="17" spans="1:17" ht="12" customHeight="1">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="28"/>
+      <c r="B17" s="29"/>
       <c r="C17" s="16" t="s">
         <v>44</v>
       </c>
@@ -1453,10 +1414,10 @@
       <c r="Q17" s="4"/>
     </row>
     <row r="18" spans="1:17" ht="12" customHeight="1">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="B18" s="28"/>
+      <c r="B18" s="29"/>
       <c r="C18" s="16" t="s">
         <v>46</v>
       </c>
@@ -1476,10 +1437,10 @@
       <c r="Q18" s="4"/>
     </row>
     <row r="19" spans="1:17" ht="12" customHeight="1">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="28"/>
+      <c r="B19" s="29"/>
       <c r="C19" s="16" t="s">
         <v>48</v>
       </c>
@@ -1499,10 +1460,10 @@
       <c r="Q19" s="4"/>
     </row>
     <row r="20" spans="1:17" ht="12" customHeight="1">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="28"/>
+      <c r="B20" s="29"/>
       <c r="C20" s="16" t="s">
         <v>50</v>
       </c>
@@ -1541,15 +1502,15 @@
       <c r="Q21" s="4"/>
     </row>
     <row r="22" spans="1:17" ht="12" customHeight="1">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
-      <c r="G22" s="29"/>
+      <c r="B22" s="32"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
@@ -1647,15 +1608,15 @@
       <c r="Q25" s="4"/>
     </row>
     <row r="26" spans="1:17" ht="12" customHeight="1">
-      <c r="A26" s="29" t="s">
+      <c r="A26" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="B26" s="29"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="29"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="32"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
@@ -1668,17 +1629,17 @@
       <c r="Q26" s="4"/>
     </row>
     <row r="27" spans="1:17" ht="12" customHeight="1">
-      <c r="A27" s="25" t="s">
+      <c r="A27" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="B27" s="25"/>
-      <c r="C27" s="26" t="s">
+      <c r="B27" s="30"/>
+      <c r="C27" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
@@ -1691,17 +1652,17 @@
       <c r="Q27" s="4"/>
     </row>
     <row r="28" spans="1:17" ht="12" customHeight="1">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26" t="s">
+      <c r="B28" s="30"/>
+      <c r="C28" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
@@ -1734,11 +1695,11 @@
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1"/>
     <row r="31" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A31" s="27" t="s">
+      <c r="A31" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="B31" s="27"/>
-      <c r="C31" s="27"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" customHeight="1">
       <c r="A32" s="18" t="s">
@@ -2742,21 +2703,6 @@
     <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C28:G28"/>
     <mergeCell ref="A31:C31"/>
@@ -2766,6 +2712,21 @@
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="C27:G27"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -2777,25 +2738,25 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M1000"/>
-  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="21.08203125" customWidth="1"/>
-    <col min="2" max="2" width="21.58203125" customWidth="1"/>
+    <col min="1" max="1" width="21.125" customWidth="1"/>
+    <col min="2" max="2" width="21.625" customWidth="1"/>
     <col min="3" max="3" width="69" customWidth="1"/>
     <col min="4" max="6" width="10.75" customWidth="1"/>
-    <col min="7" max="13" width="10.33203125" customWidth="1"/>
+    <col min="7" max="13" width="10.375" customWidth="1"/>
     <col min="14" max="26" width="11" customWidth="1"/>
     <col min="27" max="1025" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="12" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
@@ -3858,27 +3819,27 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="46.58203125" customWidth="1"/>
+    <col min="4" max="4" width="46.625" customWidth="1"/>
     <col min="5" max="6" width="10.75" customWidth="1"/>
-    <col min="7" max="14" width="10.33203125" customWidth="1"/>
+    <col min="7" max="14" width="10.375" customWidth="1"/>
     <col min="15" max="26" width="11" customWidth="1"/>
     <col min="27" max="1025" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="32" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -4945,19 +4906,19 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O1000"/>
-  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
     <col min="2" max="2" width="14.75" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="3" max="3" width="25.375" customWidth="1"/>
     <col min="4" max="4" width="37.5" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.875" customWidth="1"/>
     <col min="6" max="6" width="31.25" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
     <col min="8" max="8" width="22.75" customWidth="1"/>
-    <col min="9" max="15" width="10.33203125" customWidth="1"/>
+    <col min="9" max="15" width="10.375" customWidth="1"/>
     <col min="16" max="26" width="11" customWidth="1"/>
     <col min="27" max="1025" width="10.5" customWidth="1"/>
   </cols>
@@ -6052,30 +6013,30 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P1000"/>
-  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="2" width="16.58203125" customWidth="1"/>
+    <col min="1" max="2" width="16.625" customWidth="1"/>
     <col min="3" max="3" width="11" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="22.75" customWidth="1"/>
-    <col min="6" max="6" width="20.58203125" customWidth="1"/>
+    <col min="6" max="6" width="20.625" customWidth="1"/>
     <col min="7" max="7" width="10.75" customWidth="1"/>
-    <col min="8" max="16" width="10.33203125" customWidth="1"/>
+    <col min="8" max="16" width="10.375" customWidth="1"/>
     <col min="17" max="27" width="11" customWidth="1"/>
     <col min="28" max="1025" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="12" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
@@ -6139,22 +6100,22 @@
     </row>
     <row r="4" spans="1:16" ht="12" customHeight="1">
       <c r="A4" s="18" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="B4" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" s="35" t="s">
         <v>117</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="D4" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="E4" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="F4" s="19" t="s">
         <v>120</v>
-      </c>
-      <c r="F4" s="19" t="s">
-        <v>121</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -7178,27 +7139,27 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="46.58203125" customWidth="1"/>
+    <col min="4" max="4" width="46.625" customWidth="1"/>
     <col min="5" max="6" width="10.75" customWidth="1"/>
-    <col min="7" max="14" width="10.33203125" customWidth="1"/>
+    <col min="7" max="14" width="10.375" customWidth="1"/>
     <col min="15" max="26" width="11" customWidth="1"/>
     <col min="27" max="1025" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="29" t="s">
-        <v>108</v>
-      </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="A1" s="32" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -7218,7 +7179,7 @@
         <v>81</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D2" s="21" t="s">
         <v>66</v>
@@ -7236,12 +7197,12 @@
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
       <c r="A3" s="19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
       <c r="D3" s="19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
@@ -8265,24 +8226,24 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O1000"/>
-  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
     <col min="2" max="2" width="14.75" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="3" max="3" width="25.375" customWidth="1"/>
     <col min="4" max="4" width="37.5" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="23.58203125" customWidth="1"/>
-    <col min="7" max="15" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="15.875" customWidth="1"/>
+    <col min="6" max="6" width="23.625" customWidth="1"/>
+    <col min="7" max="15" width="10.375" customWidth="1"/>
     <col min="16" max="26" width="11" customWidth="1"/>
     <col min="27" max="1025" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
       <c r="A1" s="33" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
@@ -8307,7 +8268,7 @@
         <v>81</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D2" s="21" t="s">
         <v>89</v>
@@ -8316,7 +8277,7 @@
         <v>90</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -8330,16 +8291,16 @@
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
       <c r="A3" s="19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
       <c r="D3" s="19"/>
       <c r="E3" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="F3" s="19" t="s">
         <v>115</v>
-      </c>
-      <c r="F3" s="19" t="s">
-        <v>116</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>

</xml_diff>

<commit_message>
POCOR-5227: code enhancement in Institution > performance > report card | Status: Done
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/umairah/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{266F5220-3794-6345-ADF4-4CF848854156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4505"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="16380" windowHeight="8200" tabRatio="500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="495" windowWidth="16380" windowHeight="8205" tabRatio="500" firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -21,7 +15,7 @@
     <sheet name="Outcome Subject Comments" sheetId="6" r:id="rId6"/>
     <sheet name="Outcome Results" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -41,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="128">
   <si>
     <t>${"image":{"displayValue":"Institutions.logo_content","imageWidth":"100","imageMarginLeft":"20","imageMarginTop":"5"}}</t>
   </si>
@@ -410,12 +404,27 @@
   </si>
   <si>
     <t>Institution Subjects</t>
+  </si>
+  <si>
+    <t>Teacher Commented OpenemisNo</t>
+  </si>
+  <si>
+    <t>Teacher Commented Name</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionStudentsReportCardsComments.security_user_openemis_no","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "InstitutionStudentsReportCardsComments.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionStudentsReportCardsComments.security_user_name","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "InstitutionStudentsReportCardsComments.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "SubjectTeacher.name","rows": {"matchFrom": "SubjectTeacher.education_subject_id","matchTo": "SubjectTeacher.education_subject_id"}}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="7">
     <font>
       <sz val="12"/>
@@ -537,36 +546,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -631,7 +612,32 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -762,7 +768,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -814,7 +820,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1008,762 +1014,762 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q999"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="27.6640625" customWidth="1"/>
+    <col min="1" max="1" width="16.625" customWidth="1"/>
+    <col min="2" max="2" width="14.375" customWidth="1"/>
+    <col min="3" max="3" width="15.625" customWidth="1"/>
+    <col min="4" max="4" width="15.875" customWidth="1"/>
+    <col min="5" max="5" width="27.625" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="8" max="17" width="10.33203125" customWidth="1"/>
+    <col min="8" max="17" width="10.375" customWidth="1"/>
     <col min="18" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" customHeight="1">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A2" s="10"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="9" t="s">
+      <c r="A2" s="31"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
     </row>
     <row r="3" spans="1:17" ht="22.5" customHeight="1">
-      <c r="A3" s="10"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
+      <c r="A3" s="31"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="12" customHeight="1">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="18" t="s">
+      <c r="C5" s="30"/>
+      <c r="D5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="20"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="14"/>
-      <c r="P5" s="14"/>
-      <c r="Q5" s="14"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
     </row>
     <row r="6" spans="1:17" ht="12" customHeight="1">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="18" t="s">
+      <c r="C6" s="30"/>
+      <c r="D6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="20"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
-      <c r="L6" s="14"/>
-      <c r="M6" s="14"/>
-      <c r="N6" s="14"/>
-      <c r="O6" s="14"/>
-      <c r="P6" s="14"/>
-      <c r="Q6" s="14"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
     </row>
     <row r="7" spans="1:17" ht="12" customHeight="1">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="22" t="s">
+      <c r="C7" s="30"/>
+      <c r="D7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="23"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="14"/>
-      <c r="M7" s="14"/>
-      <c r="N7" s="14"/>
-      <c r="O7" s="14"/>
-      <c r="P7" s="14"/>
-      <c r="Q7" s="14"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
     </row>
     <row r="8" spans="1:17" ht="12" customHeight="1">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="22" t="s">
+      <c r="C8" s="30"/>
+      <c r="D8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="23"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
     </row>
     <row r="9" spans="1:17" ht="12" customHeight="1">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="22" t="s">
+      <c r="C9" s="30"/>
+      <c r="D9" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="14"/>
-      <c r="L9" s="14"/>
-      <c r="M9" s="14"/>
-      <c r="N9" s="14"/>
-      <c r="O9" s="14"/>
-      <c r="P9" s="14"/>
-      <c r="Q9" s="14"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
     </row>
     <row r="10" spans="1:17" ht="12" customHeight="1">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="22" t="s">
+      <c r="C10" s="30"/>
+      <c r="D10" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
-      <c r="M10" s="14"/>
-      <c r="N10" s="14"/>
-      <c r="O10" s="14"/>
-      <c r="P10" s="14"/>
-      <c r="Q10" s="14"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
     </row>
     <row r="11" spans="1:17" ht="12" customHeight="1">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="22" t="s">
+      <c r="C11" s="30"/>
+      <c r="D11" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="23"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="14"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="14"/>
-      <c r="N11" s="14"/>
-      <c r="O11" s="14"/>
-      <c r="P11" s="14"/>
-      <c r="Q11" s="14"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
     </row>
     <row r="12" spans="1:17" ht="12" customHeight="1">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="22" t="s">
+      <c r="C12" s="30"/>
+      <c r="D12" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="23"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="14"/>
-      <c r="N12" s="14"/>
-      <c r="O12" s="14"/>
-      <c r="P12" s="14"/>
-      <c r="Q12" s="14"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
     </row>
     <row r="13" spans="1:17" ht="12" customHeight="1">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="22" t="s">
+      <c r="C13" s="30"/>
+      <c r="D13" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="23"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="14"/>
-      <c r="M13" s="14"/>
-      <c r="N13" s="14"/>
-      <c r="O13" s="14"/>
-      <c r="P13" s="14"/>
-      <c r="Q13" s="14"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
     </row>
     <row r="14" spans="1:17" ht="12" customHeight="1">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="22" t="s">
+      <c r="C14" s="30"/>
+      <c r="D14" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="F14" s="23"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
-      <c r="M14" s="14"/>
-      <c r="N14" s="14"/>
-      <c r="O14" s="14"/>
-      <c r="P14" s="14"/>
-      <c r="Q14" s="14"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
     </row>
     <row r="15" spans="1:17" ht="16.5" customHeight="1">
-      <c r="A15" s="24"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="14"/>
-      <c r="N15" s="14"/>
-      <c r="O15" s="14"/>
-      <c r="P15" s="14"/>
-      <c r="Q15" s="14"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
     </row>
     <row r="16" spans="1:17" ht="12" customHeight="1">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="14"/>
-      <c r="P16" s="14"/>
-      <c r="Q16" s="14"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
     </row>
     <row r="17" spans="1:17" ht="12" customHeight="1">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="26" t="s">
+      <c r="B17" s="28"/>
+      <c r="C17" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
-      <c r="N17" s="14"/>
-      <c r="O17" s="14"/>
-      <c r="P17" s="14"/>
-      <c r="Q17" s="14"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
+      <c r="Q17" s="4"/>
     </row>
     <row r="18" spans="1:17" ht="12" customHeight="1">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="26" t="s">
+      <c r="B18" s="28"/>
+      <c r="C18" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="14"/>
-      <c r="N18" s="14"/>
-      <c r="O18" s="14"/>
-      <c r="P18" s="14"/>
-      <c r="Q18" s="14"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
     </row>
     <row r="19" spans="1:17" ht="12" customHeight="1">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="26" t="s">
+      <c r="B19" s="28"/>
+      <c r="C19" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="14"/>
-      <c r="M19" s="14"/>
-      <c r="N19" s="14"/>
-      <c r="O19" s="14"/>
-      <c r="P19" s="14"/>
-      <c r="Q19" s="14"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
     </row>
     <row r="20" spans="1:17" ht="12" customHeight="1">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="26" t="s">
+      <c r="B20" s="28"/>
+      <c r="C20" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14"/>
-      <c r="L20" s="14"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="14"/>
-      <c r="O20" s="14"/>
-      <c r="P20" s="14"/>
-      <c r="Q20" s="14"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
     </row>
     <row r="21" spans="1:17" ht="16.5" customHeight="1">
-      <c r="A21" s="24"/>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
-      <c r="M21" s="14"/>
-      <c r="N21" s="14"/>
-      <c r="O21" s="14"/>
-      <c r="P21" s="14"/>
-      <c r="Q21" s="14"/>
+      <c r="A21" s="14"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+      <c r="Q21" s="4"/>
     </row>
     <row r="22" spans="1:17" ht="12" customHeight="1">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
-      <c r="M22" s="14"/>
-      <c r="N22" s="14"/>
-      <c r="O22" s="14"/>
-      <c r="P22" s="14"/>
-      <c r="Q22" s="14"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
+      <c r="Q22" s="4"/>
     </row>
     <row r="23" spans="1:17" ht="12" customHeight="1">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="28" t="s">
+      <c r="D23" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="28" t="s">
+      <c r="E23" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F23" s="28" t="s">
+      <c r="F23" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="G23" s="28" t="s">
+      <c r="G23" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="14"/>
-      <c r="L23" s="14"/>
-      <c r="M23" s="14"/>
-      <c r="N23" s="14"/>
-      <c r="O23" s="14"/>
-      <c r="P23" s="14"/>
-      <c r="Q23" s="14"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="4"/>
+      <c r="Q23" s="4"/>
     </row>
     <row r="24" spans="1:17" ht="12" customHeight="1">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B24" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="D24" s="29" t="s">
+      <c r="D24" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="E24" s="29" t="s">
+      <c r="E24" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="F24" s="29" t="s">
+      <c r="F24" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="G24" s="29" t="s">
+      <c r="G24" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-      <c r="N24" s="14"/>
-      <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
-      <c r="Q24" s="14"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
     </row>
     <row r="25" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A25" s="24"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="14"/>
-      <c r="M25" s="14"/>
-      <c r="N25" s="14"/>
-      <c r="O25" s="14"/>
-      <c r="P25" s="14"/>
-      <c r="Q25" s="14"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
+      <c r="Q25" s="4"/>
     </row>
     <row r="26" spans="1:17" ht="12" customHeight="1">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
-      <c r="L26" s="14"/>
-      <c r="M26" s="14"/>
-      <c r="N26" s="14"/>
-      <c r="O26" s="14"/>
-      <c r="P26" s="14"/>
-      <c r="Q26" s="14"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="4"/>
+      <c r="Q26" s="4"/>
     </row>
     <row r="27" spans="1:17" ht="12" customHeight="1">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="B27" s="4"/>
-      <c r="C27" s="3" t="s">
+      <c r="B27" s="25"/>
+      <c r="C27" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
-      <c r="L27" s="14"/>
-      <c r="M27" s="14"/>
-      <c r="N27" s="14"/>
-      <c r="O27" s="14"/>
-      <c r="P27" s="14"/>
-      <c r="Q27" s="14"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="4"/>
+      <c r="Q27" s="4"/>
     </row>
     <row r="28" spans="1:17" ht="12" customHeight="1">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="B28" s="4"/>
-      <c r="C28" s="3" t="s">
+      <c r="B28" s="25"/>
+      <c r="C28" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="14"/>
-      <c r="K28" s="14"/>
-      <c r="L28" s="14"/>
-      <c r="M28" s="14"/>
-      <c r="N28" s="14"/>
-      <c r="O28" s="14"/>
-      <c r="P28" s="14"/>
-      <c r="Q28" s="14"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+      <c r="O28" s="4"/>
+      <c r="P28" s="4"/>
+      <c r="Q28" s="4"/>
     </row>
     <row r="29" spans="1:17" ht="12" customHeight="1">
-      <c r="A29" s="14"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="14"/>
-      <c r="J29" s="14"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="14"/>
-      <c r="M29" s="14"/>
-      <c r="N29" s="14"/>
-      <c r="O29" s="14"/>
-      <c r="P29" s="14"/>
-      <c r="Q29" s="14"/>
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
+      <c r="P29" s="4"/>
+      <c r="Q29" s="4"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1"/>
     <row r="31" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B32" s="28" t="s">
+      <c r="B32" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="18" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A33" s="29" t="s">
+      <c r="A33" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="B33" s="29" t="s">
+      <c r="B33" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C33" s="29" t="s">
+      <c r="C33" s="19" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A34" s="30"/>
-      <c r="B34" s="30"/>
+      <c r="A34" s="20"/>
+      <c r="B34" s="20"/>
     </row>
     <row r="35" spans="1:3" ht="15.75" customHeight="1">
-      <c r="B35" s="30"/>
+      <c r="B35" s="20"/>
     </row>
     <row r="36" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A36" s="28" t="s">
+      <c r="A36" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="B36" s="29" t="s">
+      <c r="B36" s="19" t="s">
         <v>78</v>
       </c>
     </row>
@@ -2732,6 +2738,21 @@
     <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C28:G28"/>
     <mergeCell ref="A31:C31"/>
@@ -2741,21 +2762,6 @@
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="C27:G27"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -2767,74 +2773,74 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="21.1640625" customWidth="1"/>
-    <col min="2" max="2" width="21.6640625" customWidth="1"/>
+    <col min="1" max="1" width="21.125" customWidth="1"/>
+    <col min="2" max="2" width="21.625" customWidth="1"/>
     <col min="3" max="3" width="69" customWidth="1"/>
-    <col min="4" max="6" width="10.6640625" customWidth="1"/>
-    <col min="7" max="13" width="10.33203125" customWidth="1"/>
+    <col min="4" max="6" width="10.625" customWidth="1"/>
+    <col min="7" max="13" width="10.375" customWidth="1"/>
     <col min="14" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="12" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
     </row>
     <row r="2" spans="1:13" ht="12" customHeight="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
     </row>
     <row r="3" spans="1:13" ht="12" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="33" t="s">
+      <c r="B3" s="19"/>
+      <c r="C3" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
     </row>
     <row r="4" spans="1:13" ht="12" customHeight="1"/>
     <row r="5" spans="1:13" ht="12" customHeight="1"/>
@@ -3847,80 +3853,80 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="46.6640625" customWidth="1"/>
-    <col min="5" max="6" width="10.6640625" customWidth="1"/>
-    <col min="7" max="14" width="10.33203125" customWidth="1"/>
+    <col min="4" max="4" width="46.625" customWidth="1"/>
+    <col min="5" max="6" width="10.625" customWidth="1"/>
+    <col min="7" max="14" width="10.375" customWidth="1"/>
     <col min="15" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
     </row>
     <row r="2" spans="1:14" ht="12" customHeight="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="D2" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29" t="s">
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="12" customHeight="1"/>
     <row r="5" spans="1:14" ht="12" customHeight="1"/>
@@ -4933,100 +4939,100 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
+    <col min="2" max="2" width="14.625" customWidth="1"/>
+    <col min="3" max="3" width="25.375" customWidth="1"/>
     <col min="4" max="4" width="37.5" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="31.1640625" customWidth="1"/>
+    <col min="5" max="5" width="15.875" customWidth="1"/>
+    <col min="6" max="6" width="31.125" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
-    <col min="8" max="8" width="22.6640625" customWidth="1"/>
-    <col min="9" max="15" width="10.33203125" customWidth="1"/>
+    <col min="8" max="8" width="22.625" customWidth="1"/>
+    <col min="9" max="15" width="10.375" customWidth="1"/>
     <col min="16" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" ht="12" customHeight="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="D2" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="E2" s="31" t="s">
+      <c r="E2" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="F2" s="31" t="s">
+      <c r="F2" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="G2" s="31" t="s">
+      <c r="G2" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="H2" s="31" t="s">
+      <c r="H2" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29" t="s">
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="F3" s="29" t="s">
+      <c r="F3" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="G3" s="29" t="s">
+      <c r="G3" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="H3" s="29" t="s">
+      <c r="H3" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
     </row>
     <row r="4" spans="1:15" ht="12" customHeight="1"/>
     <row r="5" spans="1:15" ht="12" customHeight="1"/>
@@ -6039,122 +6045,134 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="2" width="16.6640625" customWidth="1"/>
+    <col min="1" max="2" width="16.625" customWidth="1"/>
     <col min="3" max="3" width="11" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="22.6640625" customWidth="1"/>
-    <col min="6" max="6" width="20.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" customWidth="1"/>
-    <col min="8" max="16" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="22.625" customWidth="1"/>
+    <col min="6" max="6" width="20.625" customWidth="1"/>
+    <col min="7" max="7" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.75" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="16" width="10.375" customWidth="1"/>
     <col min="17" max="27" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="12" customHeight="1">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="34" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
     </row>
     <row r="3" spans="1:17" ht="12" customHeight="1">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="24" t="s">
         <v>122</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="F3" s="28" t="s">
+      <c r="F3" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
+      <c r="H3" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
     </row>
     <row r="4" spans="1:17" ht="12" customHeight="1">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="D4" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="E4" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="E4" s="29" t="s">
+      <c r="F4" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="F4" s="29" t="s">
+      <c r="G4" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
+      <c r="H4" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="12" customHeight="1"/>
     <row r="6" spans="1:17" ht="12" customHeight="1"/>
@@ -7158,7 +7176,7 @@
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -7167,80 +7185,80 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="46.6640625" customWidth="1"/>
-    <col min="5" max="6" width="10.6640625" customWidth="1"/>
-    <col min="7" max="14" width="10.33203125" customWidth="1"/>
+    <col min="4" max="4" width="46.625" customWidth="1"/>
+    <col min="5" max="6" width="10.625" customWidth="1"/>
+    <col min="7" max="14" width="10.375" customWidth="1"/>
     <col min="15" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
     </row>
     <row r="2" spans="1:14" ht="12" customHeight="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="D2" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29" t="s">
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="12" customHeight="1"/>
     <row r="5" spans="1:14" ht="12" customHeight="1"/>
@@ -8253,90 +8271,90 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
+    <col min="2" max="2" width="14.625" customWidth="1"/>
+    <col min="3" max="3" width="25.375" customWidth="1"/>
     <col min="4" max="4" width="37.5" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="23.6640625" customWidth="1"/>
-    <col min="7" max="15" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="15.875" customWidth="1"/>
+    <col min="6" max="6" width="23.625" customWidth="1"/>
+    <col min="7" max="15" width="10.375" customWidth="1"/>
     <col min="16" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" ht="12" customHeight="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="D2" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="E2" s="31" t="s">
+      <c r="E2" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="F2" s="31" t="s">
+      <c r="F2" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29" t="s">
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="F3" s="29" t="s">
+      <c r="F3" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
     </row>
     <row r="4" spans="1:15" ht="12" customHeight="1"/>
     <row r="5" spans="1:15" ht="12" customHeight="1"/>

</xml_diff>

<commit_message>
POCOR-7031: Template update STATUS:Done
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11108"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ehteramahmad/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621FD50E-19DA-7246-8274-C15B7E266AE7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4505"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="495" windowWidth="16380" windowHeight="8205" tabRatio="500" firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -21,7 +15,7 @@
     <sheet name="Outcome Subject Comments" sheetId="6" r:id="rId6"/>
     <sheet name="Outcome Results" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,6 +24,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -40,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="128">
   <si>
     <t>${"image":{"displayValue":"Institutions.logo_content","imageWidth":"100","imageMarginLeft":"20","imageMarginTop":"5"}}</t>
   </si>
@@ -99,6 +94,9 @@
     <t>Principal:</t>
   </si>
   <si>
+    <t>${Principal.user.name}</t>
+  </si>
+  <si>
     <t>Nationality:</t>
   </si>
   <si>
@@ -120,6 +118,9 @@
     <t>Homeroom Teacher:</t>
   </si>
   <si>
+    <t>${InstitutionClasses.staff.name}</t>
+  </si>
+  <si>
     <t>Date of Birth:</t>
   </si>
   <si>
@@ -405,16 +406,25 @@
     <t>Institution Subjects</t>
   </si>
   <si>
-    <t xml:space="preserve">${Principal.user.name}, ${Principal.user.preferred_name}	</t>
-  </si>
-  <si>
-    <t>${InstitutionClasses.staff.name},${InstitutionClasses.staff.preferred_name}</t>
+    <t>Teacher Commented OpenemisNo</t>
+  </si>
+  <si>
+    <t>Teacher Commented Name</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionStudentsReportCardsComments.security_user_openemis_no","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "InstitutionStudentsReportCardsComments.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionStudentsReportCardsComments.security_user_name","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "InstitutionStudentsReportCardsComments.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "SubjectTeacher.name","rows": {"matchFrom": "SubjectTeacher.education_subject_id","matchTo": "SubjectTeacher.education_subject_id"}}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="7">
     <font>
       <sz val="12"/>
@@ -536,7 +546,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -601,9 +611,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -761,7 +768,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -813,7 +820,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1007,29 +1014,29 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q999"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="27.6640625" customWidth="1"/>
+    <col min="1" max="1" width="16.625" customWidth="1"/>
+    <col min="2" max="2" width="14.375" customWidth="1"/>
+    <col min="3" max="3" width="15.625" customWidth="1"/>
+    <col min="4" max="4" width="15.875" customWidth="1"/>
+    <col min="5" max="5" width="27.625" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="8" max="17" width="10.33203125" customWidth="1"/>
+    <col min="8" max="17" width="10.375" customWidth="1"/>
     <col min="18" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
@@ -1050,14 +1057,14 @@
       <c r="Q1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A2" s="32"/>
+      <c r="A2" s="31"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
       <c r="G2" s="5"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -1071,7 +1078,7 @@
       <c r="Q2" s="4"/>
     </row>
     <row r="3" spans="1:17" ht="22.5" customHeight="1">
-      <c r="A3" s="32"/>
+      <c r="A3" s="31"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1112,10 +1119,10 @@
       <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="31"/>
+      <c r="C5" s="30"/>
       <c r="D5" s="8" t="s">
         <v>4</v>
       </c>
@@ -1139,10 +1146,10 @@
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="31"/>
+      <c r="C6" s="30"/>
       <c r="D6" s="8" t="s">
         <v>8</v>
       </c>
@@ -1166,10 +1173,10 @@
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="31"/>
+      <c r="C7" s="30"/>
       <c r="D7" s="12" t="s">
         <v>12</v>
       </c>
@@ -1193,10 +1200,10 @@
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="31"/>
+      <c r="C8" s="30"/>
       <c r="D8" s="12" t="s">
         <v>16</v>
       </c>
@@ -1220,15 +1227,15 @@
       <c r="A9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C9" s="31"/>
+      <c r="B9" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="30"/>
       <c r="D9" s="12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F9" s="13"/>
       <c r="G9" s="4"/>
@@ -1245,17 +1252,17 @@
     </row>
     <row r="10" spans="1:17" ht="12" customHeight="1">
       <c r="A10" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="31"/>
+      <c r="B10" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="30"/>
       <c r="D10" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F10" s="13"/>
       <c r="G10" s="4"/>
@@ -1272,17 +1279,17 @@
     </row>
     <row r="11" spans="1:17" ht="12" customHeight="1">
       <c r="A11" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="31" t="s">
-        <v>122</v>
-      </c>
-      <c r="C11" s="31"/>
+        <v>26</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="30"/>
       <c r="D11" s="12" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F11" s="13"/>
       <c r="G11" s="4"/>
@@ -1299,17 +1306,17 @@
     </row>
     <row r="12" spans="1:17" ht="12" customHeight="1">
       <c r="A12" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="31"/>
+        <v>30</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="30"/>
       <c r="D12" s="12" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="4"/>
@@ -1326,17 +1333,17 @@
     </row>
     <row r="13" spans="1:17" ht="12" customHeight="1">
       <c r="A13" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="31" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" s="31"/>
+        <v>34</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="30"/>
       <c r="D13" s="12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="4"/>
@@ -1353,17 +1360,17 @@
     </row>
     <row r="14" spans="1:17" ht="12" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="31"/>
+        <v>38</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="30"/>
       <c r="D14" s="12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F14" s="13"/>
       <c r="G14" s="4"/>
@@ -1398,11 +1405,11 @@
       <c r="Q15" s="4"/>
     </row>
     <row r="16" spans="1:17" ht="12" customHeight="1">
-      <c r="A16" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
+      <c r="A16" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
       <c r="D16" s="15"/>
       <c r="E16" s="15"/>
       <c r="F16" s="15"/>
@@ -1419,12 +1426,12 @@
       <c r="Q16" s="4"/>
     </row>
     <row r="17" spans="1:17" ht="12" customHeight="1">
-      <c r="A17" s="29" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" s="29"/>
+      <c r="A17" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="28"/>
       <c r="C17" s="16" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D17" s="17"/>
       <c r="E17" s="17"/>
@@ -1442,12 +1449,12 @@
       <c r="Q17" s="4"/>
     </row>
     <row r="18" spans="1:17" ht="12" customHeight="1">
-      <c r="A18" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="29"/>
+      <c r="A18" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="28"/>
       <c r="C18" s="16" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D18" s="17"/>
       <c r="E18" s="17"/>
@@ -1465,12 +1472,12 @@
       <c r="Q18" s="4"/>
     </row>
     <row r="19" spans="1:17" ht="12" customHeight="1">
-      <c r="A19" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" s="29"/>
+      <c r="A19" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="28"/>
       <c r="C19" s="16" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D19" s="17"/>
       <c r="E19" s="17"/>
@@ -1488,12 +1495,12 @@
       <c r="Q19" s="4"/>
     </row>
     <row r="20" spans="1:17" ht="12" customHeight="1">
-      <c r="A20" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="B20" s="29"/>
+      <c r="A20" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="28"/>
       <c r="C20" s="16" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D20" s="17"/>
       <c r="E20" s="17"/>
@@ -1530,15 +1537,15 @@
       <c r="Q21" s="4"/>
     </row>
     <row r="22" spans="1:17" ht="12" customHeight="1">
-      <c r="A22" s="30" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
+      <c r="A22" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
@@ -1552,25 +1559,25 @@
     </row>
     <row r="23" spans="1:17" ht="12" customHeight="1">
       <c r="A23" s="18" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G23" s="18" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -1585,25 +1592,25 @@
     </row>
     <row r="24" spans="1:17" ht="12" customHeight="1">
       <c r="A24" s="19" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
@@ -1636,15 +1643,15 @@
       <c r="Q25" s="4"/>
     </row>
     <row r="26" spans="1:17" ht="12" customHeight="1">
-      <c r="A26" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="B26" s="30"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30"/>
+      <c r="A26" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
@@ -1657,17 +1664,17 @@
       <c r="Q26" s="4"/>
     </row>
     <row r="27" spans="1:17" ht="12" customHeight="1">
-      <c r="A27" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="B27" s="26"/>
-      <c r="C27" s="27" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
+      <c r="A27" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="B27" s="25"/>
+      <c r="C27" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
@@ -1680,17 +1687,17 @@
       <c r="Q27" s="4"/>
     </row>
     <row r="28" spans="1:17" ht="12" customHeight="1">
-      <c r="A28" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="27"/>
+      <c r="A28" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
@@ -1723,32 +1730,32 @@
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1"/>
     <row r="31" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A31" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
+      <c r="A31" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" customHeight="1">
       <c r="A32" s="18" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15.75" customHeight="1">
       <c r="A33" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="15.75" customHeight="1">
@@ -1760,10 +1767,10 @@
     </row>
     <row r="36" spans="1:3" ht="15.75" customHeight="1">
       <c r="A36" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="15.75" customHeight="1"/>
@@ -2766,24 +2773,24 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="21.1640625" customWidth="1"/>
-    <col min="2" max="2" width="21.6640625" customWidth="1"/>
+    <col min="1" max="1" width="21.125" customWidth="1"/>
+    <col min="2" max="2" width="21.625" customWidth="1"/>
     <col min="3" max="3" width="69" customWidth="1"/>
-    <col min="4" max="6" width="10.6640625" customWidth="1"/>
-    <col min="7" max="13" width="10.33203125" customWidth="1"/>
+    <col min="4" max="6" width="10.625" customWidth="1"/>
+    <col min="7" max="13" width="10.375" customWidth="1"/>
     <col min="14" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="12" customHeight="1">
-      <c r="A1" s="30" t="s">
-        <v>77</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="A1" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
@@ -2797,13 +2804,13 @@
     </row>
     <row r="2" spans="1:13" ht="12" customHeight="1">
       <c r="A2" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -2818,11 +2825,11 @@
     </row>
     <row r="3" spans="1:13" ht="12" customHeight="1">
       <c r="A3" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
@@ -3846,26 +3853,26 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="46.6640625" customWidth="1"/>
-    <col min="5" max="6" width="10.6640625" customWidth="1"/>
-    <col min="7" max="14" width="10.33203125" customWidth="1"/>
+    <col min="4" max="4" width="46.625" customWidth="1"/>
+    <col min="5" max="6" width="10.625" customWidth="1"/>
+    <col min="7" max="14" width="10.375" customWidth="1"/>
     <col min="15" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
+      <c r="A1" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -3879,16 +3886,16 @@
     </row>
     <row r="2" spans="1:14" ht="12" customHeight="1">
       <c r="A2" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
@@ -3903,12 +3910,12 @@
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
       <c r="A3" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
       <c r="D3" s="19" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
@@ -4932,33 +4939,33 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
+    <col min="2" max="2" width="14.625" customWidth="1"/>
+    <col min="3" max="3" width="25.375" customWidth="1"/>
     <col min="4" max="4" width="37.5" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="31.1640625" customWidth="1"/>
+    <col min="5" max="5" width="15.875" customWidth="1"/>
+    <col min="6" max="6" width="31.125" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
-    <col min="8" max="8" width="22.6640625" customWidth="1"/>
-    <col min="9" max="15" width="10.33203125" customWidth="1"/>
+    <col min="8" max="8" width="22.625" customWidth="1"/>
+    <col min="9" max="15" width="10.375" customWidth="1"/>
     <col min="16" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
+      <c r="A1" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
       <c r="K1" s="4"/>
@@ -4969,28 +4976,28 @@
     </row>
     <row r="2" spans="1:15" ht="12" customHeight="1">
       <c r="A2" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G2" s="21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H2" s="21" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
@@ -5002,22 +5009,22 @@
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
       <c r="A3" s="19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
       <c r="D3" s="19"/>
       <c r="E3" s="19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G3" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H3" s="19" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
@@ -6038,29 +6045,31 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="2" width="16.6640625" customWidth="1"/>
+    <col min="1" max="2" width="16.625" customWidth="1"/>
     <col min="3" max="3" width="11" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="22.6640625" customWidth="1"/>
-    <col min="6" max="6" width="20.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" customWidth="1"/>
-    <col min="8" max="16" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="22.625" customWidth="1"/>
+    <col min="6" max="6" width="20.625" customWidth="1"/>
+    <col min="7" max="7" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.75" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="16" width="10.375" customWidth="1"/>
     <col min="17" max="27" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12" customHeight="1">
-      <c r="A1" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="A1" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
@@ -6073,14 +6082,14 @@
       <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="12" customHeight="1">
-      <c r="A2" s="35" t="s">
-        <v>98</v>
-      </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
+      <c r="A2" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -6094,28 +6103,32 @@
     </row>
     <row r="3" spans="1:17" ht="12" customHeight="1">
       <c r="A3" s="24" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>103</v>
-      </c>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+        <v>105</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>124</v>
+      </c>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
@@ -6126,27 +6139,33 @@
       <c r="Q3" s="4"/>
     </row>
     <row r="4" spans="1:17" ht="12" customHeight="1">
-      <c r="A4" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>105</v>
-      </c>
-      <c r="C4" s="25" t="s">
+      <c r="A4" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="B4" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="C4" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="D4" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="E4" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
+      <c r="F4" s="23" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>126</v>
+      </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
@@ -7157,7 +7176,7 @@
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -7166,26 +7185,26 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="46.6640625" customWidth="1"/>
-    <col min="5" max="6" width="10.6640625" customWidth="1"/>
-    <col min="7" max="14" width="10.33203125" customWidth="1"/>
+    <col min="4" max="4" width="46.625" customWidth="1"/>
+    <col min="5" max="6" width="10.625" customWidth="1"/>
+    <col min="7" max="14" width="10.375" customWidth="1"/>
     <col min="15" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="30" t="s">
-        <v>110</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
+      <c r="A1" s="29" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -7199,16 +7218,16 @@
     </row>
     <row r="2" spans="1:14" ht="12" customHeight="1">
       <c r="A2" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
@@ -7223,12 +7242,12 @@
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
       <c r="A3" s="19" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
       <c r="D3" s="19" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
@@ -8252,29 +8271,29 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
+    <col min="2" max="2" width="14.625" customWidth="1"/>
+    <col min="3" max="3" width="25.375" customWidth="1"/>
     <col min="4" max="4" width="37.5" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="23.6640625" customWidth="1"/>
-    <col min="7" max="15" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="15.875" customWidth="1"/>
+    <col min="6" max="6" width="23.625" customWidth="1"/>
+    <col min="7" max="15" width="10.375" customWidth="1"/>
     <col min="16" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="A1" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
@@ -8287,22 +8306,22 @@
     </row>
     <row r="2" spans="1:15" ht="12" customHeight="1">
       <c r="A2" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -8316,16 +8335,16 @@
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
       <c r="A3" s="19" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
       <c r="D3" s="19"/>
       <c r="E3" s="19" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>

</xml_diff>

<commit_message>
POCOR-7033: Develop gender placeholder in student report card STATUS:Done
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11108"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/umairah/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ehteramahmad/Sites/testingPurpose/repositories/pocor/pocor-openemis-core/webroot/export/customexcel/default_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{266F5220-3794-6345-ADF4-4CF848854156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E193C2D5-6C7D-5842-89B8-E80C5BD3ABA7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="16380" windowHeight="8200" tabRatio="500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -21,18 +21,8 @@
     <sheet name="Outcome Subject Comments" sheetId="6" r:id="rId6"/>
     <sheet name="Outcome Results" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
     </ext>
@@ -41,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="128">
   <si>
     <t>${"image":{"displayValue":"Institutions.logo_content","imageWidth":"100","imageMarginLeft":"20","imageMarginTop":"5"}}</t>
   </si>
@@ -100,9 +90,6 @@
     <t>Principal:</t>
   </si>
   <si>
-    <t>${Principal.user.name}</t>
-  </si>
-  <si>
     <t>Nationality:</t>
   </si>
   <si>
@@ -124,9 +111,6 @@
     <t>Homeroom Teacher:</t>
   </si>
   <si>
-    <t>${InstitutionClasses.staff.name}</t>
-  </si>
-  <si>
     <t>Date of Birth:</t>
   </si>
   <si>
@@ -410,6 +394,27 @@
   </si>
   <si>
     <t>Institution Subjects</t>
+  </si>
+  <si>
+    <t>Teacher Commented OpenemisNo</t>
+  </si>
+  <si>
+    <t>Teacher Commented Name</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionStudentsReportCardsComments.security_user_openemis_no","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "InstitutionStudentsReportCardsComments.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "InstitutionStudentsReportCardsComments.security_user_name","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "InstitutionStudentsReportCardsComments.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "SubjectTeacher.name","rows": {"matchFrom": "SubjectTeacher.education_subject_id","matchTo": "SubjectTeacher.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>${Principal.user.name}, ${Principal.user.preferred_name}, ${Principal.user.gender_id}</t>
+  </si>
+  <si>
+    <t>${InstitutionClasses.staff.name},${InstitutionClasses.staff.preferred_name},${InstitutionClasses.staff.gender_id}</t>
   </si>
 </sst>
 </file>
@@ -537,36 +542,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -631,7 +608,32 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -762,7 +764,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -814,7 +816,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1030,741 +1032,741 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" customHeight="1">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A2" s="10"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="9" t="s">
+      <c r="A2" s="25"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
     </row>
     <row r="3" spans="1:17" ht="22.5" customHeight="1">
-      <c r="A3" s="10"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
+      <c r="A3" s="25"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="12" customHeight="1">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="18" t="s">
+      <c r="C5" s="27"/>
+      <c r="D5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="20"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="14"/>
-      <c r="P5" s="14"/>
-      <c r="Q5" s="14"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
     </row>
     <row r="6" spans="1:17" ht="12" customHeight="1">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="18" t="s">
+      <c r="C6" s="27"/>
+      <c r="D6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="20"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
-      <c r="L6" s="14"/>
-      <c r="M6" s="14"/>
-      <c r="N6" s="14"/>
-      <c r="O6" s="14"/>
-      <c r="P6" s="14"/>
-      <c r="Q6" s="14"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
     </row>
     <row r="7" spans="1:17" ht="12" customHeight="1">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="22" t="s">
+      <c r="C7" s="27"/>
+      <c r="D7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="23"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="14"/>
-      <c r="M7" s="14"/>
-      <c r="N7" s="14"/>
-      <c r="O7" s="14"/>
-      <c r="P7" s="14"/>
-      <c r="Q7" s="14"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
     </row>
     <row r="8" spans="1:17" ht="12" customHeight="1">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="22" t="s">
+      <c r="C8" s="27"/>
+      <c r="D8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="23"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
     </row>
     <row r="9" spans="1:17" ht="12" customHeight="1">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="27"/>
+      <c r="D9" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="22" t="s">
+      <c r="E9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="14"/>
-      <c r="L9" s="14"/>
-      <c r="M9" s="14"/>
-      <c r="N9" s="14"/>
-      <c r="O9" s="14"/>
-      <c r="P9" s="14"/>
-      <c r="Q9" s="14"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
     </row>
     <row r="10" spans="1:17" ht="12" customHeight="1">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="27"/>
+      <c r="D10" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="22" t="s">
+      <c r="E10" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
-      <c r="M10" s="14"/>
-      <c r="N10" s="14"/>
-      <c r="O10" s="14"/>
-      <c r="P10" s="14"/>
-      <c r="Q10" s="14"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
     </row>
     <row r="11" spans="1:17" ht="12" customHeight="1">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" s="27"/>
+      <c r="D11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="E11" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" s="23"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="14"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="14"/>
-      <c r="N11" s="14"/>
-      <c r="O11" s="14"/>
-      <c r="P11" s="14"/>
-      <c r="Q11" s="14"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
     </row>
     <row r="12" spans="1:17" ht="12" customHeight="1">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="27"/>
+      <c r="D12" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="E12" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="F12" s="23"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="14"/>
-      <c r="N12" s="14"/>
-      <c r="O12" s="14"/>
-      <c r="P12" s="14"/>
-      <c r="Q12" s="14"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
     </row>
     <row r="13" spans="1:17" ht="12" customHeight="1">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="27"/>
+      <c r="D13" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="E13" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" s="23"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="14"/>
-      <c r="M13" s="14"/>
-      <c r="N13" s="14"/>
-      <c r="O13" s="14"/>
-      <c r="P13" s="14"/>
-      <c r="Q13" s="14"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
     </row>
     <row r="14" spans="1:17" ht="12" customHeight="1">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="27"/>
+      <c r="D14" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="E14" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="F14" s="23"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
-      <c r="M14" s="14"/>
-      <c r="N14" s="14"/>
-      <c r="O14" s="14"/>
-      <c r="P14" s="14"/>
-      <c r="Q14" s="14"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
     </row>
     <row r="15" spans="1:17" ht="16.5" customHeight="1">
-      <c r="A15" s="24"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="14"/>
-      <c r="N15" s="14"/>
-      <c r="O15" s="14"/>
-      <c r="P15" s="14"/>
-      <c r="Q15" s="14"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
     </row>
     <row r="16" spans="1:17" ht="12" customHeight="1">
-      <c r="A16" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="14"/>
-      <c r="P16" s="14"/>
-      <c r="Q16" s="14"/>
+      <c r="A16" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
     </row>
     <row r="17" spans="1:17" ht="12" customHeight="1">
-      <c r="A17" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
-      <c r="N17" s="14"/>
-      <c r="O17" s="14"/>
-      <c r="P17" s="14"/>
-      <c r="Q17" s="14"/>
+      <c r="A17" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="29"/>
+      <c r="C17" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
+      <c r="Q17" s="4"/>
     </row>
     <row r="18" spans="1:17" ht="12" customHeight="1">
-      <c r="A18" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="14"/>
-      <c r="N18" s="14"/>
-      <c r="O18" s="14"/>
-      <c r="P18" s="14"/>
-      <c r="Q18" s="14"/>
+      <c r="A18" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="29"/>
+      <c r="C18" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
     </row>
     <row r="19" spans="1:17" ht="12" customHeight="1">
-      <c r="A19" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="14"/>
-      <c r="M19" s="14"/>
-      <c r="N19" s="14"/>
-      <c r="O19" s="14"/>
-      <c r="P19" s="14"/>
-      <c r="Q19" s="14"/>
+      <c r="A19" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="29"/>
+      <c r="C19" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
     </row>
     <row r="20" spans="1:17" ht="12" customHeight="1">
-      <c r="A20" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14"/>
-      <c r="L20" s="14"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="14"/>
-      <c r="O20" s="14"/>
-      <c r="P20" s="14"/>
-      <c r="Q20" s="14"/>
+      <c r="A20" s="29" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="29"/>
+      <c r="C20" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
     </row>
     <row r="21" spans="1:17" ht="16.5" customHeight="1">
-      <c r="A21" s="24"/>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
-      <c r="M21" s="14"/>
-      <c r="N21" s="14"/>
-      <c r="O21" s="14"/>
-      <c r="P21" s="14"/>
-      <c r="Q21" s="14"/>
+      <c r="A21" s="14"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+      <c r="Q21" s="4"/>
     </row>
     <row r="22" spans="1:17" ht="12" customHeight="1">
-      <c r="A22" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
-      <c r="M22" s="14"/>
-      <c r="N22" s="14"/>
-      <c r="O22" s="14"/>
-      <c r="P22" s="14"/>
-      <c r="Q22" s="14"/>
+      <c r="A22" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="32"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
+      <c r="Q22" s="4"/>
     </row>
     <row r="23" spans="1:17" ht="12" customHeight="1">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="D23" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="E23" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="28" t="s">
+      <c r="F23" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="28" t="s">
+      <c r="G23" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F23" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="G23" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="14"/>
-      <c r="L23" s="14"/>
-      <c r="M23" s="14"/>
-      <c r="N23" s="14"/>
-      <c r="O23" s="14"/>
-      <c r="P23" s="14"/>
-      <c r="Q23" s="14"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="4"/>
+      <c r="Q23" s="4"/>
     </row>
     <row r="24" spans="1:17" ht="12" customHeight="1">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="D24" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="E24" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="D24" s="29" t="s">
+      <c r="F24" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="E24" s="29" t="s">
+      <c r="G24" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="F24" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="G24" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-      <c r="N24" s="14"/>
-      <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
-      <c r="Q24" s="14"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
     </row>
     <row r="25" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A25" s="24"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="14"/>
-      <c r="M25" s="14"/>
-      <c r="N25" s="14"/>
-      <c r="O25" s="14"/>
-      <c r="P25" s="14"/>
-      <c r="Q25" s="14"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
+      <c r="Q25" s="4"/>
     </row>
     <row r="26" spans="1:17" ht="12" customHeight="1">
-      <c r="A26" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
-      <c r="L26" s="14"/>
-      <c r="M26" s="14"/>
-      <c r="N26" s="14"/>
-      <c r="O26" s="14"/>
-      <c r="P26" s="14"/>
-      <c r="Q26" s="14"/>
+      <c r="A26" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="4"/>
+      <c r="Q26" s="4"/>
     </row>
     <row r="27" spans="1:17" ht="12" customHeight="1">
-      <c r="A27" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B27" s="4"/>
-      <c r="C27" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
-      <c r="L27" s="14"/>
-      <c r="M27" s="14"/>
-      <c r="N27" s="14"/>
-      <c r="O27" s="14"/>
-      <c r="P27" s="14"/>
-      <c r="Q27" s="14"/>
+      <c r="A27" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="B27" s="30"/>
+      <c r="C27" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="4"/>
+      <c r="Q27" s="4"/>
     </row>
     <row r="28" spans="1:17" ht="12" customHeight="1">
-      <c r="A28" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B28" s="4"/>
-      <c r="C28" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="14"/>
-      <c r="K28" s="14"/>
-      <c r="L28" s="14"/>
-      <c r="M28" s="14"/>
-      <c r="N28" s="14"/>
-      <c r="O28" s="14"/>
-      <c r="P28" s="14"/>
-      <c r="Q28" s="14"/>
+      <c r="A28" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="B28" s="30"/>
+      <c r="C28" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+      <c r="O28" s="4"/>
+      <c r="P28" s="4"/>
+      <c r="Q28" s="4"/>
     </row>
     <row r="29" spans="1:17" ht="12" customHeight="1">
-      <c r="A29" s="14"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="14"/>
-      <c r="J29" s="14"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="14"/>
-      <c r="M29" s="14"/>
-      <c r="N29" s="14"/>
-      <c r="O29" s="14"/>
-      <c r="P29" s="14"/>
-      <c r="Q29" s="14"/>
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
+      <c r="P29" s="4"/>
+      <c r="Q29" s="4"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1"/>
     <row r="31" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A31" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
+      <c r="A31" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A32" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="B32" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="C32" s="28" t="s">
-        <v>73</v>
+      <c r="A32" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A33" s="29" t="s">
+      <c r="A33" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="19" t="s">
         <v>74</v>
-      </c>
-      <c r="B33" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="C33" s="29" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A34" s="30"/>
-      <c r="B34" s="30"/>
+      <c r="A34" s="20"/>
+      <c r="B34" s="20"/>
     </row>
     <row r="35" spans="1:3" ht="15.75" customHeight="1">
-      <c r="B35" s="30"/>
+      <c r="B35" s="20"/>
     </row>
     <row r="36" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A36" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="B36" s="29" t="s">
-        <v>78</v>
+      <c r="A36" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="15.75" customHeight="1"/>
@@ -2780,61 +2782,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="12" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
+      <c r="A1" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
     </row>
     <row r="2" spans="1:13" ht="12" customHeight="1">
-      <c r="A2" s="31" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
+      <c r="A2" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
     </row>
     <row r="3" spans="1:13" ht="12" customHeight="1">
-      <c r="A3" s="29" t="s">
-        <v>82</v>
-      </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="33" t="s">
-        <v>83</v>
-      </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
+      <c r="A3" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="19"/>
+      <c r="C3" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
     </row>
     <row r="4" spans="1:13" ht="12" customHeight="1"/>
     <row r="5" spans="1:13" ht="12" customHeight="1"/>
@@ -3861,66 +3863,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
+      <c r="A1" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
     </row>
     <row r="2" spans="1:14" ht="12" customHeight="1">
-      <c r="A2" s="31" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>85</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
+      <c r="A2" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
-      <c r="A3" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
+      <c r="A3" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="12" customHeight="1"/>
     <row r="5" spans="1:14" ht="12" customHeight="1"/>
@@ -4950,83 +4952,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
+      <c r="A1" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" ht="12" customHeight="1">
-      <c r="A2" s="31" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>85</v>
-      </c>
-      <c r="D2" s="31" t="s">
+      <c r="A2" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="E2" s="31" t="s">
+      <c r="G2" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="F2" s="31" t="s">
+      <c r="H2" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="G2" s="31" t="s">
-        <v>92</v>
-      </c>
-      <c r="H2" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29" t="s">
+      <c r="G3" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="F3" s="29" t="s">
+      <c r="H3" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="G3" s="29" t="s">
-        <v>97</v>
-      </c>
-      <c r="H3" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
     </row>
     <row r="4" spans="1:15" ht="12" customHeight="1"/>
     <row r="5" spans="1:15" ht="12" customHeight="1"/>
@@ -6048,113 +6050,125 @@
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="22.6640625" customWidth="1"/>
     <col min="6" max="6" width="20.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" customWidth="1"/>
-    <col min="8" max="16" width="10.33203125" customWidth="1"/>
+    <col min="7" max="7" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.6640625" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="16" width="10.33203125" customWidth="1"/>
     <col min="17" max="27" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
+      <c r="A1" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="12" customHeight="1">
-      <c r="A2" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
+      <c r="A2" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
     </row>
     <row r="3" spans="1:17" ht="12" customHeight="1">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="I3" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="B3" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="C3" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="D3" s="28" t="s">
-        <v>102</v>
-      </c>
-      <c r="E3" s="28" t="s">
-        <v>103</v>
-      </c>
-      <c r="F3" s="28" t="s">
-        <v>104</v>
-      </c>
-      <c r="G3" s="28" t="s">
-        <v>105</v>
-      </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
     </row>
     <row r="4" spans="1:17" ht="12" customHeight="1">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="E4" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="F4" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="G4" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="E4" s="29" t="s">
-        <v>110</v>
-      </c>
-      <c r="F4" s="29" t="s">
-        <v>111</v>
-      </c>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
+      <c r="H4" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="12" customHeight="1"/>
     <row r="6" spans="1:17" ht="12" customHeight="1"/>
@@ -7158,7 +7172,7 @@
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -7181,66 +7195,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
+      <c r="A1" s="32" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
     </row>
     <row r="2" spans="1:14" ht="12" customHeight="1">
-      <c r="A2" s="31" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
+      <c r="A2" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
-      <c r="A3" s="29" t="s">
-        <v>114</v>
-      </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29" t="s">
-        <v>115</v>
-      </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
+      <c r="A3" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="12" customHeight="1"/>
     <row r="5" spans="1:14" ht="12" customHeight="1"/>
@@ -8268,75 +8282,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
+      <c r="A1" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" ht="12" customHeight="1">
-      <c r="A2" s="31" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>89</v>
-      </c>
-      <c r="E2" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="F2" s="31" t="s">
-        <v>117</v>
-      </c>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
+      <c r="A2" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="F3" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29" t="s">
-        <v>119</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>120</v>
-      </c>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
     </row>
     <row r="4" spans="1:15" ht="12" customHeight="1"/>
     <row r="5" spans="1:15" ht="12" customHeight="1"/>

</xml_diff>

<commit_message>
POCOR-5054: code enahnce for showing modified user in report_card_template | Status: Done
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="128">
   <si>
     <t>${"image":{"displayValue":"Institutions.logo_content","imageWidth":"100","imageMarginLeft":"20","imageMarginTop":"5"}}</t>
   </si>
@@ -415,13 +415,16 @@
   </si>
   <si>
     <t>${"match": {"displayValue": "InstitutionStudentsReportCardsComments.security_user_name","rows": {"matchFrom": "AssessmentItems.education_subject_id","matchTo": "InstitutionStudentsReportCardsComments.education_subject_id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "AssessmentItemResults.marks_formatted","type":"number","format":"2","rows": {"matchFrom": "InstitutionSubjectStudentsWithName.education_subject_id","matchTo": "AssessmentItemResults.education_subject_id"},"columns": {"matchFrom": "AssessmentPeriods.id","matchTo": "AssessmentItemResults.assessment_period_id"}}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -469,6 +472,12 @@
     </font>
     <font>
       <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -549,7 +558,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -627,6 +636,9 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -646,8 +658,8 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1291,10 +1303,10 @@
       <c r="A11" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="29" t="s">
         <v>122</v>
       </c>
-      <c r="C11" s="36"/>
+      <c r="C11" s="29"/>
       <c r="D11" s="12" t="s">
         <v>26</v>
       </c>
@@ -1415,11 +1427,11 @@
       <c r="Q15" s="4"/>
     </row>
     <row r="16" spans="1:17" ht="12" customHeight="1">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
       <c r="D16" s="15"/>
       <c r="E16" s="15"/>
       <c r="F16" s="15"/>
@@ -1436,10 +1448,10 @@
       <c r="Q16" s="4"/>
     </row>
     <row r="17" spans="1:17" ht="12" customHeight="1">
-      <c r="A17" s="30" t="s">
+      <c r="A17" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="30"/>
+      <c r="B17" s="31"/>
       <c r="C17" s="16" t="s">
         <v>42</v>
       </c>
@@ -1459,10 +1471,10 @@
       <c r="Q17" s="4"/>
     </row>
     <row r="18" spans="1:17" ht="12" customHeight="1">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="30"/>
+      <c r="B18" s="31"/>
       <c r="C18" s="16" t="s">
         <v>44</v>
       </c>
@@ -1482,10 +1494,10 @@
       <c r="Q18" s="4"/>
     </row>
     <row r="19" spans="1:17" ht="12" customHeight="1">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="30"/>
+      <c r="B19" s="31"/>
       <c r="C19" s="16" t="s">
         <v>46</v>
       </c>
@@ -1505,10 +1517,10 @@
       <c r="Q19" s="4"/>
     </row>
     <row r="20" spans="1:17" ht="12" customHeight="1">
-      <c r="A20" s="30" t="s">
+      <c r="A20" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="30"/>
+      <c r="B20" s="31"/>
       <c r="C20" s="16" t="s">
         <v>48</v>
       </c>
@@ -1547,15 +1559,15 @@
       <c r="Q21" s="4"/>
     </row>
     <row r="22" spans="1:17" ht="12" customHeight="1">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="33"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
@@ -1653,15 +1665,15 @@
       <c r="Q25" s="4"/>
     </row>
     <row r="26" spans="1:17" ht="12" customHeight="1">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="33"/>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
@@ -1674,17 +1686,17 @@
       <c r="Q26" s="4"/>
     </row>
     <row r="27" spans="1:17" ht="12" customHeight="1">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="31"/>
-      <c r="C27" s="32" t="s">
+      <c r="B27" s="32"/>
+      <c r="C27" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
@@ -1697,17 +1709,17 @@
       <c r="Q27" s="4"/>
     </row>
     <row r="28" spans="1:17" ht="12" customHeight="1">
-      <c r="A28" s="31" t="s">
+      <c r="A28" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="B28" s="31"/>
-      <c r="C28" s="32" t="s">
+      <c r="B28" s="32"/>
+      <c r="C28" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
@@ -1740,11 +1752,11 @@
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1"/>
     <row r="31" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A31" s="29" t="s">
+      <c r="A31" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="29"/>
-      <c r="C31" s="29"/>
+      <c r="B31" s="30"/>
+      <c r="C31" s="30"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" customHeight="1">
       <c r="A32" s="18" t="s">
@@ -2796,11 +2808,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="12" customHeight="1">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
@@ -3877,12 +3889,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -4966,16 +4978,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
       <c r="K1" s="4"/>
@@ -6070,14 +6082,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12" customHeight="1">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
@@ -6090,14 +6102,14 @@
       <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="12" customHeight="1">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -6156,16 +6168,18 @@
       <c r="C4" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="37" t="s">
+        <v>127</v>
+      </c>
+      <c r="E4" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="F4" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="G4" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="G4" s="4"/>
       <c r="H4" s="4" t="s">
         <v>125</v>
       </c>
@@ -7205,12 +7219,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -8292,14 +8306,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>

</xml_diff>

<commit_message>
POCOR-5054: Updated xls file upload | Status: Done
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -497,7 +497,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -553,6 +553,15 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -569,7 +578,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -582,12 +591,11 @@
     <xf numFmtId="49" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -624,13 +632,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -642,7 +650,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -655,10 +663,13 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1058,7 +1069,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" customHeight="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
@@ -1079,14 +1090,14 @@
       <c r="Q1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A2" s="26"/>
+      <c r="A2" s="25"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
       <c r="G2" s="5"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -1100,7 +1111,7 @@
       <c r="Q2" s="4"/>
     </row>
     <row r="3" spans="1:17" ht="22.5" customHeight="1">
-      <c r="A3" s="26"/>
+      <c r="A3" s="25"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1141,17 +1152,16 @@
       <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="28"/>
+      <c r="C5" s="27"/>
       <c r="D5" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="10"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
@@ -1168,17 +1178,16 @@
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="28"/>
+      <c r="C6" s="27"/>
       <c r="D6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="10"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
@@ -1195,17 +1204,17 @@
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="28"/>
-      <c r="D7" s="12" t="s">
+      <c r="C7" s="27"/>
+      <c r="D7" s="11" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="13"/>
+      <c r="F7" s="12"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
@@ -1222,17 +1231,17 @@
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="12" t="s">
+      <c r="C8" s="27"/>
+      <c r="D8" s="11" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="13"/>
+      <c r="F8" s="12"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -1249,17 +1258,17 @@
       <c r="A9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="12" t="s">
+      <c r="C9" s="27"/>
+      <c r="D9" s="11" t="s">
         <v>19</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="13"/>
+      <c r="F9" s="12"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
@@ -1276,17 +1285,17 @@
       <c r="A10" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="12" t="s">
+      <c r="C10" s="27"/>
+      <c r="D10" s="11" t="s">
         <v>23</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="13"/>
+      <c r="F10" s="12"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
@@ -1303,17 +1312,17 @@
       <c r="A11" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="C11" s="29"/>
-      <c r="D11" s="12" t="s">
+      <c r="C11" s="28"/>
+      <c r="D11" s="11" t="s">
         <v>26</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="13"/>
+      <c r="F11" s="12"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
@@ -1330,17 +1339,17 @@
       <c r="A12" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="28" t="s">
+      <c r="B12" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="12" t="s">
+      <c r="C12" s="27"/>
+      <c r="D12" s="11" t="s">
         <v>30</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="13"/>
+      <c r="F12" s="12"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -1357,17 +1366,17 @@
       <c r="A13" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="28"/>
-      <c r="D13" s="12" t="s">
+      <c r="C13" s="27"/>
+      <c r="D13" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="13"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
@@ -1384,17 +1393,17 @@
       <c r="A14" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="28" t="s">
+      <c r="B14" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="12" t="s">
+      <c r="C14" s="27"/>
+      <c r="D14" s="11" t="s">
         <v>38</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="13"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -1408,13 +1417,13 @@
       <c r="Q14" s="4"/>
     </row>
     <row r="15" spans="1:17" ht="16.5" customHeight="1">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
@@ -1427,15 +1436,15 @@
       <c r="Q15" s="4"/>
     </row>
     <row r="16" spans="1:17" ht="12" customHeight="1">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
@@ -1448,17 +1457,17 @@
       <c r="Q16" s="4"/>
     </row>
     <row r="17" spans="1:17" ht="12" customHeight="1">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="31"/>
-      <c r="C17" s="16" t="s">
+      <c r="B17" s="30"/>
+      <c r="C17" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
@@ -1471,17 +1480,17 @@
       <c r="Q17" s="4"/>
     </row>
     <row r="18" spans="1:17" ht="12" customHeight="1">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="31"/>
-      <c r="C18" s="16" t="s">
+      <c r="B18" s="30"/>
+      <c r="C18" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -1494,17 +1503,17 @@
       <c r="Q18" s="4"/>
     </row>
     <row r="19" spans="1:17" ht="12" customHeight="1">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="31"/>
-      <c r="C19" s="16" t="s">
+      <c r="B19" s="30"/>
+      <c r="C19" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
@@ -1517,17 +1526,17 @@
       <c r="Q19" s="4"/>
     </row>
     <row r="20" spans="1:17" ht="12" customHeight="1">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="31"/>
-      <c r="C20" s="16" t="s">
+      <c r="B20" s="30"/>
+      <c r="C20" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
@@ -1540,13 +1549,13 @@
       <c r="Q20" s="4"/>
     </row>
     <row r="21" spans="1:17" ht="16.5" customHeight="1">
-      <c r="A21" s="14"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
@@ -1559,15 +1568,15 @@
       <c r="Q21" s="4"/>
     </row>
     <row r="22" spans="1:17" ht="12" customHeight="1">
-      <c r="A22" s="34" t="s">
+      <c r="A22" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="34"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
@@ -1580,25 +1589,25 @@
       <c r="Q22" s="4"/>
     </row>
     <row r="23" spans="1:17" ht="12" customHeight="1">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="D23" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="E23" s="18" t="s">
+      <c r="E23" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="F23" s="18" t="s">
+      <c r="F23" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="G23" s="18" t="s">
+      <c r="G23" s="17" t="s">
         <v>56</v>
       </c>
       <c r="H23" s="4"/>
@@ -1613,25 +1622,25 @@
       <c r="Q23" s="4"/>
     </row>
     <row r="24" spans="1:17" ht="12" customHeight="1">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="C24" s="19" t="s">
+      <c r="C24" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="D24" s="19" t="s">
+      <c r="D24" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E24" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="19" t="s">
+      <c r="F24" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="G24" s="19" t="s">
+      <c r="G24" s="18" t="s">
         <v>63</v>
       </c>
       <c r="H24" s="4"/>
@@ -1646,13 +1655,13 @@
       <c r="Q24" s="4"/>
     </row>
     <row r="25" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A25" s="14"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
       <c r="J25" s="4"/>
@@ -1665,15 +1674,15 @@
       <c r="Q25" s="4"/>
     </row>
     <row r="26" spans="1:17" ht="12" customHeight="1">
-      <c r="A26" s="34" t="s">
+      <c r="A26" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="34"/>
+      <c r="B26" s="33"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
@@ -1686,17 +1695,17 @@
       <c r="Q26" s="4"/>
     </row>
     <row r="27" spans="1:17" ht="12" customHeight="1">
-      <c r="A27" s="32" t="s">
+      <c r="A27" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="33" t="s">
+      <c r="B27" s="31"/>
+      <c r="C27" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
@@ -1709,17 +1718,17 @@
       <c r="Q27" s="4"/>
     </row>
     <row r="28" spans="1:17" ht="12" customHeight="1">
-      <c r="A28" s="32" t="s">
+      <c r="A28" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="33" t="s">
+      <c r="B28" s="31"/>
+      <c r="C28" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
@@ -1752,46 +1761,46 @@
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1"/>
     <row r="31" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A31" s="30" t="s">
+      <c r="A31" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="30"/>
-      <c r="C31" s="30"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A32" s="18" t="s">
+      <c r="A32" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B32" s="18" t="s">
+      <c r="B32" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="17" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="B33" s="19" t="s">
+      <c r="B33" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="C33" s="19" t="s">
+      <c r="C33" s="18" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A34" s="20"/>
-      <c r="B34" s="20"/>
+      <c r="A34" s="19"/>
+      <c r="B34" s="19"/>
     </row>
     <row r="35" spans="1:3" ht="15.75" customHeight="1">
-      <c r="B35" s="20"/>
+      <c r="B35" s="19"/>
     </row>
     <row r="36" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A36" s="18" t="s">
+      <c r="A36" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="B36" s="19" t="s">
+      <c r="B36" s="18" t="s">
         <v>76</v>
       </c>
     </row>
@@ -2808,11 +2817,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="12" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
@@ -2825,13 +2834,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2" spans="1:13" ht="12" customHeight="1">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>64</v>
       </c>
       <c r="D2" s="4"/>
@@ -2846,11 +2855,11 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3" spans="1:13" ht="12" customHeight="1">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="23" t="s">
+      <c r="B3" s="18"/>
+      <c r="C3" s="22" t="s">
         <v>81</v>
       </c>
       <c r="D3" s="4"/>
@@ -3889,12 +3898,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -3907,16 +3916,16 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2" spans="1:14" ht="12" customHeight="1">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>64</v>
       </c>
       <c r="E2" s="4"/>
@@ -3931,12 +3940,12 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19" t="s">
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18" t="s">
         <v>85</v>
       </c>
       <c r="E3" s="4"/>
@@ -4978,16 +4987,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
       <c r="K1" s="4"/>
@@ -4997,28 +5006,28 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" ht="12" customHeight="1">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>91</v>
       </c>
       <c r="I2" s="4"/>
@@ -5030,22 +5039,22 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19" t="s">
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="18" t="s">
         <v>96</v>
       </c>
       <c r="I3" s="4"/>
@@ -6085,14 +6094,14 @@
       <c r="A1" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
       <c r="J1" s="4"/>
       <c r="K1" s="4"/>
       <c r="L1" s="4"/>
@@ -6105,14 +6114,14 @@
       <c r="A2" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
@@ -6122,31 +6131,31 @@
       <c r="P2" s="4"/>
     </row>
     <row r="3" spans="1:17" ht="12" customHeight="1">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="I3" s="18" t="s">
+      <c r="I3" s="17" t="s">
         <v>124</v>
       </c>
       <c r="J3" s="4"/>
@@ -6159,25 +6168,25 @@
       <c r="Q3" s="4"/>
     </row>
     <row r="4" spans="1:17" ht="12" customHeight="1">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="24" t="s">
         <v>127</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>108</v>
       </c>
       <c r="H4" s="4" t="s">
@@ -7192,8 +7201,8 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -7219,12 +7228,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -7237,16 +7246,16 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2" spans="1:14" ht="12" customHeight="1">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>64</v>
       </c>
       <c r="E2" s="4"/>
@@ -7261,12 +7270,12 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3" spans="1:14" ht="12" customHeight="1">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19" t="s">
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18" t="s">
         <v>112</v>
       </c>
       <c r="E3" s="4"/>
@@ -8306,14 +8315,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="34" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
@@ -8325,22 +8334,22 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" ht="12" customHeight="1">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>114</v>
       </c>
       <c r="G2" s="4"/>
@@ -8354,16 +8363,16 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" ht="12" customHeight="1">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19" t="s">
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>117</v>
       </c>
       <c r="G3" s="4"/>

</xml_diff>

<commit_message>
POCOR-7424: Deleted empty three rows in excel, status:done
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -646,7 +646,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -787,14 +787,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -901,7 +893,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q1048576"/>
-  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.37"/>
@@ -1738,48 +1730,39 @@
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="26"/>
-      <c r="B44" s="26"/>
+      <c r="A44" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="B44" s="35"/>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="35"/>
-      <c r="B45" s="36"/>
+      <c r="A45" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="B45" s="26" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="35"/>
-      <c r="B46" s="36"/>
+      <c r="A46" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="B46" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" s="36"/>
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="37" t="s">
-        <v>92</v>
-      </c>
-      <c r="B47" s="37"/>
+      <c r="A47" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="B47" s="33" t="s">
+        <v>97</v>
+      </c>
     </row>
-    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="B48" s="26" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="27" t="s">
-        <v>94</v>
-      </c>
-      <c r="B49" s="33" t="s">
-        <v>95</v>
-      </c>
-      <c r="C49" s="38"/>
-    </row>
-    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="B50" s="33" t="s">
-        <v>97</v>
-      </c>
-    </row>
+    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2726,9 +2709,9 @@
     <row r="994" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="995" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="996" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="997" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="998" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="999" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="26">
@@ -2757,7 +2740,7 @@
     <mergeCell ref="C29:G29"/>
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A44:B44"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
@@ -2775,7 +2758,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M1000"/>
-  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.62"/>
@@ -2803,13 +2786,13 @@
       <c r="M1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="35" t="s">
         <v>68</v>
       </c>
       <c r="D2" s="5"/>
@@ -2828,7 +2811,7 @@
         <v>101</v>
       </c>
       <c r="B3" s="27"/>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="38" t="s">
         <v>102</v>
       </c>
       <c r="D3" s="5"/>
@@ -3859,7 +3842,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17"/>
@@ -3889,16 +3872,16 @@
       <c r="N1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="35" t="s">
         <v>104</v>
       </c>
-      <c r="D2" s="37" t="s">
+      <c r="D2" s="35" t="s">
         <v>68</v>
       </c>
       <c r="E2" s="5"/>
@@ -4949,7 +4932,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O1000"/>
-  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.63"/>
@@ -4983,28 +4966,28 @@
       <c r="O1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="35" t="s">
         <v>104</v>
       </c>
-      <c r="D2" s="37" t="s">
+      <c r="D2" s="35" t="s">
         <v>108</v>
       </c>
-      <c r="E2" s="37" t="s">
+      <c r="E2" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="F2" s="37" t="s">
+      <c r="F2" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="G2" s="37" t="s">
+      <c r="G2" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="H2" s="37" t="s">
+      <c r="H2" s="35" t="s">
         <v>112</v>
       </c>
       <c r="I2" s="5"/>
@@ -6059,7 +6042,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q1000"/>
-  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="16.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
@@ -6092,17 +6075,17 @@
       <c r="P1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="39" t="s">
         <v>119</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
@@ -6112,10 +6095,10 @@
       <c r="P2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="40" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="40" t="s">
         <v>121</v>
       </c>
       <c r="C3" s="26" t="s">
@@ -6158,7 +6141,7 @@
       <c r="C4" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="D4" s="43" t="s">
+      <c r="D4" s="41" t="s">
         <v>132</v>
       </c>
       <c r="E4" s="27" t="s">
@@ -7201,7 +7184,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17"/>
@@ -7231,16 +7214,16 @@
       <c r="N1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="D2" s="37" t="s">
+      <c r="D2" s="35" t="s">
         <v>68</v>
       </c>
       <c r="E2" s="5"/>
@@ -8291,7 +8274,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O1000"/>
-  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.63"/>
@@ -8323,22 +8306,22 @@
       <c r="O1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="D2" s="37" t="s">
+      <c r="D2" s="35" t="s">
         <v>108</v>
       </c>
-      <c r="E2" s="37" t="s">
+      <c r="E2" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="F2" s="37" t="s">
+      <c r="F2" s="35" t="s">
         <v>143</v>
       </c>
       <c r="G2" s="5"/>

</xml_diff>

<commit_message>
report card xlsx update||new placeholder
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="149">
   <si>
     <t xml:space="preserve">${"image":{"displayValue":"Institutions.logo_content","imageWidth":"100","imageMarginLeft":"20","imageMarginTop":"5"}}</t>
   </si>
@@ -152,6 +152,12 @@
   </si>
   <si>
     <t xml:space="preserve">${InstitutionStudentsReportCards.student.body_mass_index}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${InstitutionStudentsReportCards.gpa}</t>
   </si>
   <si>
     <t xml:space="preserve">Gender:</t>
@@ -893,7 +899,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q1048576"/>
-  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.37"/>
@@ -1254,14 +1260,18 @@
       <c r="Q14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9"/>
-      <c r="B15" s="10"/>
+      <c r="A15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>43</v>
+      </c>
       <c r="C15" s="10"/>
       <c r="D15" s="17" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F15" s="15"/>
       <c r="G15" s="19"/>
@@ -1297,7 +1307,7 @@
     </row>
     <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="20"/>
@@ -1318,11 +1328,11 @@
     </row>
     <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B18" s="22"/>
       <c r="C18" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D18" s="24"/>
       <c r="E18" s="24"/>
@@ -1341,11 +1351,11 @@
     </row>
     <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="22" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B19" s="22"/>
       <c r="C19" s="23" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D19" s="24"/>
       <c r="E19" s="24"/>
@@ -1364,11 +1374,11 @@
     </row>
     <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B20" s="22"/>
       <c r="C20" s="23" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D20" s="24"/>
       <c r="E20" s="24"/>
@@ -1387,11 +1397,11 @@
     </row>
     <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B21" s="22"/>
       <c r="C21" s="23" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D21" s="24"/>
       <c r="E21" s="24"/>
@@ -1429,7 +1439,7 @@
     </row>
     <row r="23" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="25" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B23" s="25"/>
       <c r="C23" s="25"/>
@@ -1450,25 +1460,25 @@
     </row>
     <row r="24" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="26" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C24" s="26" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
@@ -1483,25 +1493,25 @@
     </row>
     <row r="25" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="27" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F25" s="27" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G25" s="27" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
@@ -1535,7 +1545,7 @@
     </row>
     <row r="27" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
@@ -1556,11 +1566,11 @@
     </row>
     <row r="28" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B28" s="28"/>
       <c r="C28" s="29" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D28" s="29"/>
       <c r="E28" s="29"/>
@@ -1579,11 +1589,11 @@
     </row>
     <row r="29" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="28" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B29" s="28"/>
       <c r="C29" s="29" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D29" s="29"/>
       <c r="E29" s="29"/>
@@ -1622,31 +1632,31 @@
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B32" s="20"/>
       <c r="C32" s="20"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="26" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B34" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1658,17 +1668,17 @@
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="26" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B37" s="27" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B40" s="31"/>
       <c r="C40" s="31"/>
@@ -1679,48 +1689,48 @@
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="26" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B41" s="26" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D41" s="26" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E41" s="26" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F41" s="26" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G41" s="26" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="27" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C42" s="32" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D42" s="33" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F42" s="33" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G42" s="33" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H42" s="34"/>
       <c r="I42" s="34"/>
@@ -1731,33 +1741,33 @@
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="35" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B44" s="35"/>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="26" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C46" s="36"/>
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2744,7 +2754,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -2758,19 +2768,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M1000"/>
-  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="10.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="10.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="7" style="0" width="10.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="14" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -2787,13 +2797,13 @@
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="35" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C2" s="35" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -2808,11 +2818,11 @@
     </row>
     <row r="3" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B3" s="27"/>
       <c r="C3" s="38" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -3828,7 +3838,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -3842,20 +3852,20 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="10.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="10.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="7" style="0" width="10.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="15" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -3873,16 +3883,16 @@
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="35" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C2" s="35" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D2" s="35" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -3897,12 +3907,12 @@
     </row>
     <row r="3" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B3" s="27"/>
       <c r="C3" s="27"/>
       <c r="D3" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
@@ -4918,7 +4928,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -4932,11 +4942,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O1000"/>
-  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="37.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="31.11"/>
@@ -4948,7 +4958,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="31" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B1" s="31"/>
       <c r="C1" s="31"/>
@@ -4967,28 +4977,28 @@
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="35" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C2" s="35" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D2" s="35" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E2" s="35" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H2" s="35" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
@@ -5000,22 +5010,22 @@
     </row>
     <row r="3" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B3" s="27"/>
       <c r="C3" s="27"/>
       <c r="D3" s="27"/>
       <c r="E3" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F3" s="27" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G3" s="27" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H3" s="27" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
@@ -6028,7 +6038,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -6042,21 +6052,21 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q1000"/>
-  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="16.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="8" style="0" width="10.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="17" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="31" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B1" s="31"/>
       <c r="C1" s="31"/>
@@ -6076,7 +6086,7 @@
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="39" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B2" s="39"/>
       <c r="C2" s="39"/>
@@ -6096,31 +6106,31 @@
     </row>
     <row r="3" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B3" s="40" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G3" s="26" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H3" s="26" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I3" s="26" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
@@ -6133,31 +6143,31 @@
     </row>
     <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="27" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D4" s="41" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E4" s="27" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F4" s="27" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
@@ -7170,7 +7180,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -7184,20 +7194,20 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="10.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="10.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="7" style="0" width="10.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="15" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -7215,16 +7225,16 @@
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="35" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C2" s="35" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D2" s="35" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -7239,12 +7249,12 @@
     </row>
     <row r="3" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B3" s="27"/>
       <c r="C3" s="27"/>
       <c r="D3" s="27" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
@@ -8260,7 +8270,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
@@ -8274,11 +8284,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O1000"/>
-  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="37.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.61"/>
@@ -8288,7 +8298,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="31" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B1" s="31"/>
       <c r="C1" s="31"/>
@@ -8307,22 +8317,22 @@
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="35" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C2" s="35" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D2" s="35" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E2" s="35" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
@@ -8336,16 +8346,16 @@
     </row>
     <row r="3" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B3" s="27"/>
       <c r="C3" s="27"/>
       <c r="D3" s="27"/>
       <c r="E3" s="27" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F3" s="27" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
@@ -9360,7 +9370,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Arial,Regular"&amp;10&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
POCOR-9232: working on calss and level ranking in report cards | status: In progress
</commit_message>
<xml_diff>
--- a/webroot/export/customexcel/default_templates/report_card_template.xlsx
+++ b/webroot/export/customexcel/default_templates/report_card_template.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\pocor-openemis-core\webroot\export\customexcel\default_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC350C84-2367-4EF7-B92F-3FC7F49DA0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -20,8 +21,9 @@
     <sheet name="GPA" sheetId="6" r:id="rId6"/>
     <sheet name="Outcome Subject Comments" sheetId="7" r:id="rId7"/>
     <sheet name="Outcome Results" sheetId="8" r:id="rId8"/>
+    <sheet name="Class And Level" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -31,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="187">
   <si>
     <t>${"image":{"displayValue":"Institutions.logo_content","imageWidth":"100","imageMarginLeft":"20","imageMarginTop":"5"}}</t>
   </si>
@@ -523,13 +525,82 @@
   </si>
   <si>
     <t>${InstitutionStudentsReportCards.age}</t>
+  </si>
+  <si>
+    <t>Academic Period</t>
+  </si>
+  <si>
+    <t>Institution Name</t>
+  </si>
+  <si>
+    <t>Institution Code</t>
+  </si>
+  <si>
+    <t>Class Name</t>
+  </si>
+  <si>
+    <t>Student OpenEMIS No</t>
+  </si>
+  <si>
+    <t>Student First Name</t>
+  </si>
+  <si>
+    <t>Student Last Name</t>
+  </si>
+  <si>
+    <t>Institution Subject</t>
+  </si>
+  <si>
+    <t>Total Mark</t>
+  </si>
+  <si>
+    <t>Class Ranking</t>
+  </si>
+  <si>
+    <t>Level Ranking</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.academic_period","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.institution_name","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.institution_code","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.education_grade","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.class_name","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.student_openemis_no","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.student_first_name","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.student_last_name","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.institution_subject","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.total_mark","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.class_ranking","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
+  </si>
+  <si>
+    <t>${"match": {"displayValue": "ClassAndLevelRanking.level_ranking","rows": {"matchFrom": "ClassAndLevelRanking.id","matchTo": "ClassAndLevelRanking.id"}}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="15">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="16">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -636,8 +707,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -654,6 +731,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0077D4"/>
+        <bgColor rgb="FF0077D4"/>
       </patternFill>
     </fill>
   </fills>
@@ -719,7 +802,7 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -815,23 +898,11 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -840,20 +911,33 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1199,7 +1283,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q996"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.5"/>
   <cols>
@@ -1214,7 +1298,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" customHeight="1">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
@@ -1235,14 +1319,14 @@
       <c r="Q1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A2" s="46"/>
+      <c r="A2" s="38"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="47" t="s">
+      <c r="C2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
       <c r="G2" s="5"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -1256,7 +1340,7 @@
       <c r="Q2" s="4"/>
     </row>
     <row r="3" spans="1:17" ht="22.5" customHeight="1">
-      <c r="A3" s="46"/>
+      <c r="A3" s="38"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
@@ -1297,10 +1381,10 @@
       <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="44" t="s">
+      <c r="B5" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="44"/>
+      <c r="C5" s="40"/>
       <c r="D5" s="9" t="s">
         <v>4</v>
       </c>
@@ -1323,10 +1407,10 @@
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="44"/>
+      <c r="C6" s="40"/>
       <c r="D6" s="9" t="s">
         <v>8</v>
       </c>
@@ -1349,10 +1433,10 @@
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="44"/>
+      <c r="C7" s="40"/>
       <c r="D7" s="12" t="s">
         <v>12</v>
       </c>
@@ -1376,10 +1460,10 @@
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="44"/>
+      <c r="C8" s="40"/>
       <c r="D8" s="12" t="s">
         <v>16</v>
       </c>
@@ -1403,10 +1487,10 @@
       <c r="A9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="44" t="s">
+      <c r="B9" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="44"/>
+      <c r="C9" s="40"/>
       <c r="D9" s="12" t="s">
         <v>20</v>
       </c>
@@ -1430,10 +1514,10 @@
       <c r="A10" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="44"/>
+      <c r="C10" s="40"/>
       <c r="D10" s="12" t="s">
         <v>24</v>
       </c>
@@ -1457,10 +1541,10 @@
       <c r="A11" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="45" t="s">
+      <c r="B11" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="45"/>
+      <c r="C11" s="41"/>
       <c r="D11" s="12" t="s">
         <v>28</v>
       </c>
@@ -1484,10 +1568,10 @@
       <c r="A12" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="44" t="s">
+      <c r="B12" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="44"/>
+      <c r="C12" s="40"/>
       <c r="D12" s="12" t="s">
         <v>32</v>
       </c>
@@ -1511,10 +1595,10 @@
       <c r="A13" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="44" t="s">
+      <c r="B13" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="44"/>
+      <c r="C13" s="40"/>
       <c r="D13" s="12" t="s">
         <v>36</v>
       </c>
@@ -1538,10 +1622,10 @@
       <c r="A14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="44" t="s">
+      <c r="B14" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="44"/>
+      <c r="C14" s="40"/>
       <c r="D14" s="12" t="s">
         <v>40</v>
       </c>
@@ -1608,11 +1692,11 @@
       <c r="Q16" s="4"/>
     </row>
     <row r="17" spans="1:17" ht="12" customHeight="1">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39"/>
+      <c r="B17" s="42"/>
+      <c r="C17" s="42"/>
       <c r="D17" s="17"/>
       <c r="E17" s="17"/>
       <c r="F17" s="17"/>
@@ -1629,10 +1713,10 @@
       <c r="Q17" s="4"/>
     </row>
     <row r="18" spans="1:17" ht="12" customHeight="1">
-      <c r="A18" s="42" t="s">
+      <c r="A18" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="42"/>
+      <c r="B18" s="43"/>
       <c r="C18" s="18" t="s">
         <v>48</v>
       </c>
@@ -1652,10 +1736,10 @@
       <c r="Q18" s="4"/>
     </row>
     <row r="19" spans="1:17" ht="12" customHeight="1">
-      <c r="A19" s="42" t="s">
+      <c r="A19" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="42"/>
+      <c r="B19" s="43"/>
       <c r="C19" s="18" t="s">
         <v>50</v>
       </c>
@@ -1675,10 +1759,10 @@
       <c r="Q19" s="4"/>
     </row>
     <row r="20" spans="1:17" ht="12" customHeight="1">
-      <c r="A20" s="42" t="s">
+      <c r="A20" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="B20" s="42"/>
+      <c r="B20" s="43"/>
       <c r="C20" s="18" t="s">
         <v>52</v>
       </c>
@@ -1698,10 +1782,10 @@
       <c r="Q20" s="4"/>
     </row>
     <row r="21" spans="1:17" ht="12" customHeight="1">
-      <c r="A21" s="42" t="s">
+      <c r="A21" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="B21" s="42"/>
+      <c r="B21" s="43"/>
       <c r="C21" s="18" t="s">
         <v>54</v>
       </c>
@@ -1740,15 +1824,15 @@
       <c r="Q22" s="4"/>
     </row>
     <row r="23" spans="1:17" ht="12" customHeight="1">
-      <c r="A23" s="43" t="s">
+      <c r="A23" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="43"/>
+      <c r="B23" s="44"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
@@ -1846,15 +1930,15 @@
       <c r="Q26" s="4"/>
     </row>
     <row r="27" spans="1:17" ht="12" customHeight="1">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="44" t="s">
         <v>70</v>
       </c>
-      <c r="B27" s="43"/>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
+      <c r="B27" s="44"/>
+      <c r="C27" s="44"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="44"/>
+      <c r="F27" s="44"/>
+      <c r="G27" s="44"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
@@ -1867,17 +1951,17 @@
       <c r="Q27" s="4"/>
     </row>
     <row r="28" spans="1:17" ht="12" customHeight="1">
-      <c r="A28" s="37" t="s">
+      <c r="A28" s="45" t="s">
         <v>71</v>
       </c>
-      <c r="B28" s="37"/>
-      <c r="C28" s="38" t="s">
+      <c r="B28" s="45"/>
+      <c r="C28" s="46" t="s">
         <v>72</v>
       </c>
-      <c r="D28" s="38"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="38"/>
-      <c r="G28" s="38"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="46"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
@@ -1890,17 +1974,17 @@
       <c r="Q28" s="4"/>
     </row>
     <row r="29" spans="1:17" ht="12" customHeight="1">
-      <c r="A29" s="37" t="s">
+      <c r="A29" s="45" t="s">
         <v>73</v>
       </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="38" t="s">
+      <c r="B29" s="45"/>
+      <c r="C29" s="46" t="s">
         <v>74</v>
       </c>
-      <c r="D29" s="38"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="38"/>
-      <c r="G29" s="38"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
@@ -1933,11 +2017,11 @@
     </row>
     <row r="31" spans="1:17" ht="15.75" customHeight="1"/>
     <row r="32" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="42" t="s">
         <v>75</v>
       </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
+      <c r="B32" s="42"/>
+      <c r="C32" s="42"/>
     </row>
     <row r="33" spans="1:12" ht="15.75" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -1979,15 +2063,15 @@
     <row r="38" spans="1:12" ht="15.75" customHeight="1"/>
     <row r="39" spans="1:12" ht="15.75" customHeight="1"/>
     <row r="40" spans="1:12" ht="15.75" customHeight="1">
-      <c r="A40" s="40" t="s">
+      <c r="A40" s="47" t="s">
         <v>83</v>
       </c>
-      <c r="B40" s="40"/>
-      <c r="C40" s="40"/>
-      <c r="D40" s="40"/>
-      <c r="E40" s="40"/>
-      <c r="F40" s="40"/>
-      <c r="G40" s="40"/>
+      <c r="B40" s="47"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="47"/>
+      <c r="E40" s="47"/>
+      <c r="F40" s="47"/>
+      <c r="G40" s="47"/>
     </row>
     <row r="41" spans="1:12" ht="15.75" customHeight="1">
       <c r="A41" s="20" t="s">
@@ -2042,10 +2126,10 @@
     </row>
     <row r="43" spans="1:12" ht="15.75" customHeight="1"/>
     <row r="44" spans="1:12" ht="15.75" customHeight="1">
-      <c r="A44" s="41" t="s">
+      <c r="A44" s="48" t="s">
         <v>94</v>
       </c>
-      <c r="B44" s="41"/>
+      <c r="B44" s="48"/>
     </row>
     <row r="45" spans="1:12" ht="15.75" customHeight="1">
       <c r="A45" s="20" t="s">
@@ -2073,7 +2157,7 @@
       </c>
     </row>
     <row r="48" spans="1:12" ht="15.75" customHeight="1">
-      <c r="A48" s="49" t="s">
+      <c r="A48" s="37" t="s">
         <v>162</v>
       </c>
       <c r="B48" s="24" t="s">
@@ -3030,32 +3114,32 @@
     <row r="996" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A44:B44"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A23:G23"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C28:G28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="C29:G29"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3067,7 +3151,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M1000"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.5"/>
   <cols>
@@ -3079,11 +3163,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="12" customHeight="1">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="44" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
@@ -4146,7 +4230,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N1000"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.5"/>
   <cols>
@@ -4159,12 +4243,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -5231,7 +5315,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:O1000"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.5"/>
   <cols>
@@ -5248,16 +5332,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="47" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
       <c r="K1" s="4"/>
@@ -6337,7 +6421,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:Q1000"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.5"/>
   <cols>
@@ -6351,17 +6435,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="47" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
       <c r="J1" s="4"/>
       <c r="K1" s="4"/>
       <c r="L1" s="4"/>
@@ -6371,17 +6455,17 @@
       <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:17" ht="12" customHeight="1">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="49" t="s">
         <v>121</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
@@ -7474,7 +7558,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AMJ992"/>
   <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="15.5"/>
   <cols>
@@ -9566,7 +9650,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:N1000"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.5"/>
   <cols>
@@ -9579,12 +9663,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12" customHeight="1">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="44" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -10651,7 +10735,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:O1000"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.5"/>
   <cols>
@@ -10666,14 +10750,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="47" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
@@ -11744,4 +11828,90 @@
     <oddFooter>&amp;C&amp;"Arial,Regular"&amp;10Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB87FF98-190A-41CB-AACE-A98DA7855C75}">
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="50" t="s">
+        <v>164</v>
+      </c>
+      <c r="B1" s="50" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1" s="50" t="s">
+        <v>166</v>
+      </c>
+      <c r="D1" s="50" t="s">
+        <v>142</v>
+      </c>
+      <c r="E1" s="50" t="s">
+        <v>167</v>
+      </c>
+      <c r="F1" s="50" t="s">
+        <v>168</v>
+      </c>
+      <c r="G1" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="H1" s="50" t="s">
+        <v>170</v>
+      </c>
+      <c r="I1" s="50" t="s">
+        <v>171</v>
+      </c>
+      <c r="J1" s="50" t="s">
+        <v>172</v>
+      </c>
+      <c r="K1" s="50" t="s">
+        <v>173</v>
+      </c>
+      <c r="L1" s="50" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G2" t="s">
+        <v>181</v>
+      </c>
+      <c r="H2" t="s">
+        <v>182</v>
+      </c>
+      <c r="I2" t="s">
+        <v>183</v>
+      </c>
+      <c r="J2" t="s">
+        <v>184</v>
+      </c>
+      <c r="K2" t="s">
+        <v>185</v>
+      </c>
+      <c r="L2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>